<commit_message>
refactor: prepare runtime and LLM implementation directories
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -1217,7 +1217,7 @@
       </c>
       <c r="AA4" s="5" t="inlineStr">
         <is>
-          <t>sha256:1dee7e7ce90f70c40d02907f11be7b55665495fdcaa3dfdec3ab478953c5c38c</t>
+          <t>sha256:1e23ba2952b874e8029345d74ff832663be433870e57e403ccac4370e9237916</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:570d7db5b7480c6b3a3a3adcc953158f7c496e44a79e90ad1ca3a4df676d573f</t>
+          <t>sha256:f8f1bc3e7a01d6ffd739d9fbe695e28533e4c410847a09b6405a7dbd4c2e948a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(frontend): add agent list table view
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_D5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_D2'!$A$1:$AA$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_D5'!$A$1:$AA$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -551,10 +551,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
@@ -603,25 +603,67 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>AGENT-LIST-VIEWS</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Agent list grid and table views</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Switch between the existing agent cards and a data-backed table without changing page-level content or agent operations.</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-LIST-RULE-001
+AGENT-LIST-RULE-002
+AGENT-LIST-RULE-003
+AGENT-LIST-RULE-004
+AGENT-LIST-RULE-005</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>D1
+D4</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>{"notes":"User request and same-page WeMeeting high-fidelity reference; no Edge window inspected.","requirement_ids":["AGENT-LIST-REQ-001","AGENT-LIST-REQ-002"],"spec_path":"docs/handoffs/2026-10-08-agent-list-high-fidelity.md"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Silent model retry stream visibility</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Successful model attempts stream raw content while failed attempts leave no visible or persisted fragments.</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-013
 CMSR-RULE-014
@@ -631,7 +673,7 @@
 CMSR-RULE-018</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>D1
 D2
@@ -640,14 +682,14 @@
 D5</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>{"requirement_ids":["CMSR-005"],"spec_path":"nexent-doc/docs/Developing/chat-message-model-silent-retry/proposal.md"}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -658,13 +700,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -681,7 +723,7 @@
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -830,38 +872,42 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>CMSR-D1-001</t>
+          <t>AGENT-LIST-D1-001</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>CMSR-005</t>
+          <t>AGENT-LIST-VIEWS</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>CMSR-005</t>
+          <t>AGENT-LIST-REQ-001
+AGENT-LIST-REQ-002</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>CMSR-RULE-013
-CMSR-RULE-014</t>
+          <t>AGENT-LIST-RULE-001
+AGENT-LIST-RULE-002
+AGENT-LIST-RULE-003
+AGENT-LIST-RULE-004
+AGENT-LIST-RULE-005</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Observer emits safe content before stream completion</t>
+          <t>Render table view with data-backed agent metadata</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>SDK-UT</t>
+          <t>FE-COMP</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -876,40 +922,47 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Verify bounded marker lookahead and attempt state reset.</t>
+          <t>Verify Ant Design table rendering, including header separators and content-based sizing constraints, plus columns, row data, update-time source, and action callbacks without changing the card view contract.</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Create an isolated observer and a controlled chunk sequence.</t>
+          <t>Render the table with agents containing author, tags, status, and update_time values.
+Render a second agent without update_time but with create_time.</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>{"profile":"mock","sequence":"failed partial, rollback, successful split code and think markers"}</t>
+          <t>{"no_update_agent":{"author":null,"create_time":"2026-09-17T10:30:00","update_time":null},"profile":"mock","updated_agent":{"author":"刘晨","tags":["保健"],"update_time":"2026-09-18T10:30:00"}}</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>1. Feed a safe prefix and pause the source. =&gt; The prefix is emitted before flush or commit.
-2. Roll back the first attempt and feed split markers in the second. =&gt; The second output is ordered and contains no first-attempt residue.</t>
+          <t>1. Render the table with the mocked agent rows. =&gt; The seven columns appear in the specified order in StandardTable backed by Ant Design Table; internal header columns have 1px
+2. Render a row whose update_time is absent and whose create_time is present. =&gt; The update-time cell shows the missing-value placeholder rather than the creation date.
+3. Trigger the row's detail, configure, and publish actions. =&gt; Each callback receives the corresponding agent or numeric agent ID.</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>The earliest safe content is observable before completion.
-Split markers retain their original semantics.</t>
+          <t>The table labels include 更新时间 and do not label agents as knowledge bases.
+The table is rendered through StandardTable with the documented typography, backgrounds, 40px rows,
+The table wrapper uses content-based height up to 500px and internal overflow scrolling; it is not forced to fill unused space.
+Update time is formatted from update_time only; missing or invalid timestamps do not fall back to create_time.
+Creator uses author when present and a placeholder when absent.
+The card component and its data behavior remain unchanged.</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>No stale fragment crosses attempts.
-No code is executed by the observer.</t>
+          <t>Do not modify page title, guide area, tabs, or card-mode content.
+Do not add or change backend requests or response contracts.
+Do not fabricate creator or update-time values.</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Safe prefix emitted before flush.","Raw code tag retained.","No failed-attempt residue."],"inputs":["normal content","split &lt;think&gt; and &lt;/think&gt;","raw &lt;code&gt; content"],"unit_boundary":"Observer.add_model_new_token and attempt lifecycle"}</t>
+          <t>{"assertions":["Table headers render in the required order.","Update time never falls back to create_time.","Missing creator and timestamp values render placeholders.","Action callbacks receive the correct row data.","Header separators are 14px high, vertically centered, and","The scroll wrapper is content-sized with a 500px maximum rather than flex-growing to fill unused space."],"inputs":["agent rows","locale strings","row-action callbacks"],"unit_boundary":"AgentListTable React component with mocked callbacks and translation."}</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr"/>
@@ -920,17 +973,17 @@
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>pytest</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>test/automation/d1/test_model_attempt_stream.py</t>
+          <t>test/automation/d1/run_agent_list_table_test.mjs</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>test_cmsr_d1_001</t>
+          <t>agentListTable.test.tsx</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
@@ -947,85 +1000,214 @@
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
-          <t>sha256:625e8c8829b51b9cd91344555d05c5ebfdc7bd766d8485eab99b9f22773f3233</t>
+          <t>sha256:42084a90cedb1ae8ffba7cbe7cf1411f12a57a0d42205e6580e12ad08042aeb9</t>
         </is>
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:242f1aaf8a5fe4427f503e5acb8db2cc6cb5096782c2e4fdf49fcb17ec471420</t>
+          <t>sha256:6dd34b7871a706a8b5fc3aa75f7a0dce8d785c1dbc328369e21a9b47cebef59e</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>CMSR-D1-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>CMSR-005</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>CMSR-005</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>CMSR-RULE-013
+CMSR-RULE-014</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Observer emits safe content before stream completion</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Verify bounded marker lookahead and attempt state reset.</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Create an isolated observer and a controlled chunk sequence.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock","sequence":"failed partial, rollback, successful split code and think markers"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Feed a safe prefix and pause the source. =&gt; The prefix is emitted before flush or commit.
+2. Roll back the first attempt and feed split markers in the second. =&gt; The second output is ordered and contains no first-attempt residue.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>The earliest safe content is observable before completion.
+Split markers retain their original semantics.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No stale fragment crosses attempts.
+No code is executed by the observer.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Safe prefix emitted before flush.","Raw code tag retained.","No failed-attempt residue."],"inputs":["normal content","split &lt;think&gt; and &lt;/think&gt;","raw &lt;code&gt; content"],"unit_boundary":"Observer.add_model_new_token and attempt lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_model_attempt_stream.py</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>test_cmsr_d1_001</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:625e8c8829b51b9cd91344555d05c5ebfdc7bd766d8485eab99b9f22773f3233</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:242f1aaf8a5fe4427f503e5acb8db2cc6cb5096782c2e4fdf49fcb17ec471420</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
           <t>CMSR-D1-002</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-014
 CMSR-RULE-015</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Running step labels precede reasoning and survive retry rollback</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>FE-COMP</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Verify immediate running labels, rollback preservation, legacy history and removal of terminal label-only cards.</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Create the streaming adapter with a controlled SSE fixture.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequences":["step 1, failed attempt, rollback, successful raw code, parse","legacy content before step label"]}</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>1. Emit a step label before any model content. =&gt; A running reasoning card displays Step 1 immediately.
 2. Roll back a partial attempt and stream successful raw code. =&gt; Step 1 remains during rollback and only successful raw code follows it.
 3. Parse and reload both new and legacy-order history. =&gt; One code card and one labeled nonempty reasoning card remain; a terminal label-only card is absent.</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Step label appears before first token.
 Rollback preserves the label.
@@ -1033,326 +1215,326 @@
 Old history prepends late labels.</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>No failed-attempt content.
 No duplicate code card.
 No sibling invocation mutation.</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Running label is visible before content.","Terminal label-only step is hidden.","Successful code is visible after the label before commit.","History equals live output."],"inputs":["step_count","model_attempt_control","model_output_thinking","parse"],"unit_boundary":"Frontend live and history reasoning projection"}</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="T4" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_reasoning_card.ts</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr">
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-002</t>
         </is>
       </c>
-      <c r="V3" s="5" t="inlineStr">
+      <c r="V4" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr"/>
-      <c r="X3" s="5" t="inlineStr"/>
-      <c r="Y3" s="5" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" s="5" t="inlineStr"/>
+      <c r="Y4" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z3" s="5" t="inlineStr">
+      <c r="Z4" s="5" t="inlineStr">
         <is>
           <t>sha256:b614502639e969ab0f3840d1381f1b12b01cb5b693a0b02d17387192b230b354</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="inlineStr">
+      <c r="AA4" s="5" t="inlineStr">
         <is>
           <t>sha256:03f5fae5200c76ca296c75ab0ebf225f190fb3fe6a7f52c7c8c7e0da2a97d07c</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-003</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-014
 CMSR-RULE-016</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>CoreAgent commits streamed valid semantic repair</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>A protocol-invalid first attempt rolls back while its single preceding step label survives and the corrected result streams and commits.</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>A controlled model yields an invalid response then a pausable valid code action at step one.</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequence":"invalid code, rollback, corrected code chunks, commit, parse"}</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>1. Begin step one and return protocol-invalid model content. =&gt; Exactly one step label precedes begin; the attempt rolls back and one repair is scheduled.
 2. Pause the valid repair after its first safe chunk. =&gt; That chunk is visible before model completion.
 3. Complete the repair and classify it. =&gt; Its attempt commits and a single parse follows.</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Corrected content is streamed and committed.
 Only the corrected action is executed.
 Lifecycle logs identify the repair without content.</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>No failed content after rollback.
 No repair instruction in user output.
 No suppressed successful stream.</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Step label occurs before both model attempts and only once.","Successful repair does not set stream suppression.","Corrected attempt commits once.","Invalid attempt rolls back once."],"inputs":["step one","invalid model content","valid streamed &lt;code&gt; action"],"unit_boundary":"CoreAgent semantic repair and deferred model attempt lifecycle"}</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_semantic_repair_stream.py</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U5" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_003</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V5" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr"/>
-      <c r="X4" s="5" t="inlineStr"/>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="W5" s="5" t="inlineStr"/>
+      <c r="X5" s="5" t="inlineStr"/>
+      <c r="Y5" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z4" s="5" t="inlineStr">
+      <c r="Z5" s="5" t="inlineStr">
         <is>
           <t>sha256:7ef8664f2224d068d7deafecf80f09353d734bc10b35a1147b3cc58d1ae6eacd</t>
         </is>
       </c>
-      <c r="AA4" s="5" t="inlineStr">
+      <c r="AA5" s="5" t="inlineStr">
         <is>
           <t>sha256:1dee7e7ce90f70c40d02907f11be7b55665495fdcaa3dfdec3ab478953c5c38c</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-004</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-018</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Rejected model output diagnostics distinguish budget exhaustion without default content leakage</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Correlate each protocol rejection to the model response shape and budget while gating bounded raw previews.</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Use isolated model diagnostics for a reasoning-only length response and a malformed nonempty response.</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","responses":["length with 4096 reasoning-only output tokens","malformed nonempty code Action"]}</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>1. Reject a reasoning-only length response with diagnostics disabled. =&gt; The log records model, attempt, requested and consumed tokens, reasoning and content counts, and reasoning-only budget exhaustion without raw text.
 2. Reject a malformed content response. =&gt; The distinct protocol reason and response shape are logged under its own attempt identifier.
 3. Enable diagnostic content preview for a rejected response longer than the preview cap. =&gt; Only a single escaped bounded prefix of model content and reasoning is logged; the full text remains absent.</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Each rejection is attributable to one attempt and specific failure class.
 Raw output is absent by default and bounded on explicit opt-in.</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>No model output or user prompt enters SSE or persisted history from diagnostics.
 No secret or full raw payload is logged by default.
 No retry-budget or execution behavior changes.</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Reasoning-only budget exhaustion flag is accurate.","Logs include attempt and token counts.","Default logs omit raw content.","Opt-in previews are escaped and capped."],"inputs":["finish_reason=length","reasoning_content","invalid code Action","explicit diagnostic flag"],"unit_boundary":"OpenAI model response diagnostics and CoreAgent protocol-error logging"}</t>
         </is>
       </c>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S5" s="5" t="inlineStr">
+      <c r="S6" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T5" s="5" t="inlineStr">
+      <c r="T6" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_protocol_rejection_diagnostics.py</t>
         </is>
       </c>
-      <c r="U5" s="5" t="inlineStr">
+      <c r="U6" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_004</t>
         </is>
       </c>
-      <c r="V5" s="5" t="inlineStr">
+      <c r="V6" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr"/>
-      <c r="X5" s="5" t="inlineStr"/>
-      <c r="Y5" s="5" t="inlineStr">
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z5" s="5" t="inlineStr">
+      <c r="Z6" s="5" t="inlineStr">
         <is>
           <t>sha256:9f06a6565fff8e542fdcb89725b5fc7f669ad52b07301bdc99aa3e2eba23552c</t>
         </is>
       </c>
-      <c r="AA5" s="5" t="inlineStr">
+      <c r="AA6" s="5" t="inlineStr">
         <is>
           <t>sha256:a53056127d5f2efce4a9d98c92c9c97892451de0d1d353603584612c0a9ef1ba</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA5"/>
+  <autoFilter ref="A1:AA6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1653,7 +1835,7 @@
       <c r="X2" s="5" t="inlineStr"/>
       <c r="Y2" s="5" t="inlineStr">
         <is>
-          <t>校验通过</t>
+          <t>实现哈希失效</t>
         </is>
       </c>
       <c r="Z2" s="5" t="inlineStr">
@@ -1993,12 +2175,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2013,10 +2195,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -2165,20 +2347,160 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>AGENT-LIST-D4-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-LIST-VIEWS</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-LIST-REQ-001
+AGENT-LIST-REQ-002</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-LIST-RULE-001
+AGENT-LIST-RULE-002
+AGENT-LIST-RULE-003
+AGENT-LIST-RULE-004
+AGENT-LIST-RULE-005</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Switch between the agent card and table presentations</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Verify Ant Design table separators and content-responsive sizing at desktop and constrained viewport widths, and confirm that table view retains existing list workflows.</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Open the agent list with at least two mocked agents, including one with update_time and one without it.</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>{"agent_count":8,"profile":"mock","viewport":{"height":1080,"width":1920}}</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>1. Switch from card mode to table mode. =&gt; The page heading, guide, and tabs remain unchanged while the table and its pagination appear.
+2. Verify columns and representative row values. =&gt; The column order is 名称、类型、描述、状态、创建人、更新时间、操作; timestamps reflect update_time only.
+3. Inspect the header separators and table height with eight rendered rows, then search to a single matching row. =&gt; Internal header columns have 1px
+4. Search for an agent, activate its configure action, then return and switch back to card mode. =&gt; Search and navigation still work, and the card presentation returns with its prior layout and metadata.</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>At 1920×1080 the table occupies the measured 1807px content width; its height follows its rendered rows, grows no higher than 500px, and does not fill unused space.
+The table uses StandardTable with 14px/#191919/0px typography, white rows, a
+Narrow filter headers show both the label and icon with 8px horizontal padding.
+When rows exceed the 500px cap or the available list area, scrolling stays inside the table body and pagination remains below it.
+Search, configure, publish, import, and view switching remain usable.
+Page-level content above the list and existing card mode are unchanged.</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>No backend API or data mutation is introduced by switching views.
+Do not use create_time as update_time.
+Do not add body vertical separators or an outer table border; header separators remain centered and shorter than the 40px header cell.</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>{"actor":"Agent list user","failure_evidence":["Missing/incorrect table headings or row values.","Search, navigation, pagination, or view switching fails.","The table changes content above the list or mutates agent data."],"final_business_result":["The same agent collection remains available in either presentation.","Existing list operations remain reachable."],"journey":["Open the agent list.","Switch between card and table modes.","Search and open an agent configuration."]}</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d4/run_agent_list_views_e2e.mjs</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>agent-list-high-fidelity.spec.ts</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr"/>
+      <c r="X2" s="5" t="inlineStr"/>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>sha256:1093e9eea123f868058b2922bcb8becb7058e0378301e97276df51156c4ba9fc</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>sha256:a905ec4d8fcce1e93354988f937f8f560872b64738f762662e6250e2413b9b8b</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
           <t>CMSR-D4-001</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-013
 CMSR-RULE-014
@@ -2186,48 +2508,48 @@
 CMSR-RULE-016</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Browser shows retry output incrementally without blank steps</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>E2E</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Verify a user sees only successful raw code and one executed action in a real conversation.</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>A local Nexent instance
 test tenant and controllable model provider are configured.</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequences":["failed transport partial then success","step-one invalid protocol then valid paused repair"]}</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>1. Open Agent chat and send the fixed prompt. =&gt; Step 1 appears before the first model token; the first partial output is then rolled back while the label remains.
 2. Pause the second provider response after its first safe fragment. =&gt; The reasoning card displays the successful raw fragment before provider completion.
@@ -2235,7 +2557,7 @@
 4. Repeat in a new conversation with semantic repair at step one. =&gt; Corrected raw code is visible during the pause and after refresh; Connecting does not persist.</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Running Step 1 is visible before content.
 No terminal label-only reasoning card.
@@ -2243,59 +2565,59 @@
 Refreshed history matches the final UI.</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>No failed partial text after rollback.
 No duplicate execution card.</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>{"actor":"Authenticated test tenant user","failure_evidence":["Retain browser screenshot","network timing and console trace on failure."],"final_business_result":["Only the committed attempt and its single executed code action are visible."],"journey":["Open the Agent conversation.","Trigger controlled retry.","Observe streaming.","Reload and inspect history."]}</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>{"profiles":[{"name":"mock","required_services":["model-provider"]}]}</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr"/>
-      <c r="T2" s="5" t="inlineStr"/>
-      <c r="U2" s="5" t="inlineStr"/>
-      <c r="V2" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>model-provider</t>
         </is>
       </c>
-      <c r="X2" s="5" t="inlineStr"/>
-      <c r="Y2" s="5" t="inlineStr">
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z2" s="5" t="inlineStr">
+      <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>sha256:f110f582fe091286fdaa5301f8bdc22703bf583fc7c6c95214ae8c8187a612a1</t>
         </is>
       </c>
-      <c r="AA2" s="5" t="inlineStr">
+      <c r="AA3" s="5" t="inlineStr">
         <is>
           <t>sha256:4f53cda18c2baa0c0354bb5f9a3ecbe5ed12ab4d8e11ba873c2f11161202b945</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(aidp): streamline knowledge base creation UI
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>AIDP knowledge bases are listed in a card or table overview with an independent name search, a collapsible three-step guide and a full-page file view per knowledge base; creation moves to a dedicated two-step page that carries permission, chunking, retrieval, graph and model configuration. The ES knowledge base path stays untouched.</t>
+          <t>AIDP knowledge bases are listed in a card or table overview with an independent name search, a collapsible three-step guide and a full-page file view per knowledge base; creation uses one dedicated full-page form for permissions, chunking, retrieval, graph and model configuration, submits directly, and leaves file upload to the detail page. The ES knowledge base path stays untouched.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -685,7 +685,8 @@
 AKPR-RULE-012
 AKPR-RULE-013
 AKPR-RULE-015
-AKPR-RULE-016</t>
+AKPR-RULE-016
+AKPR-RULE-017</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -2552,12 +2553,13 @@
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>AKPR-RULE-010
-AKPR-RULE-016</t>
+AKPR-RULE-016
+AKPR-RULE-017</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Creation page keeps switches beside labels and aligns paired controls</t>
+          <t>Creation page uses 18px titles and submits directly from its single form</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -2582,12 +2584,12 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Verify the AIDP create page is full-width, section controls have the designed visual grouping, and paired controls share a baseline.</t>
+          <t>Verify the AIDP create page uses the approved title sizes and single-page submit flow while keeping section controls aligned.</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Render the first creation step at desktop width with safety, graph and VLM controls visible.</t>
+          <t>Render the AIDP creation page at desktop width with a valid mock create response.</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
@@ -2597,14 +2599,18 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>1. Render the page header and form. =&gt; The creation form uses the available content width and the breadcrumb reads knowledge base / create knowledge base.
-2. Inspect safety, graph and VLM toggle groups. =&gt; Each switch sits beside its corresponding label and help icon.
-3. Inspect fields that share a row. =&gt; Both controls use the same label structure and their input or slider starts differ by no more than one pixel.</t>
+          <t>1. Render the page header and form. =&gt; The creation form uses the available content width; breadcrumb labels are 18px and no step indicator or optional upload stage is rendered.
+2. Inspect graph and VLM toggle groups. =&gt; Each switch sits beside its corresponding label and help icon.
+3. Inspect section headings and fields that share a row. =&gt; Both controls use the same label structure and their input or slider starts differ by no more than one pixel.
+4. Fill required fields and submit the create form. =&gt; One create request is sent, no upload request is sent, and success navigates to the created knowledge base detail page.
+5. Render the detail information tab for a seeded knowledge base. =&gt; The detail breadcrumb and configuration, graph and permission section headings use 18px text.</t>
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr">
         <is>
           <t>No fixed narrow modal-sized content column constrains the create page.
+The create breadcrumb title and form section headings use 18px text.
+The form creates the knowledge base directly without an intermediate step or upload stage.
 Switches are adjacent to their own labels rather than the far edge of the row.
 Paired model, chunking and retrieval controls align consistently.</t>
         </is>
@@ -2617,7 +2623,7 @@
       </c>
       <c r="P17" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["The creation header and form fill the available page content width.","Switches are grouped within 12 pixels of their labels.","Paired controls use consistent label and field alignment."],"inputs":["desktop viewport","graph toggle","VLM toggle","paired model controls"],"unit_boundary":"AIDP create form section layout and toggle grouping"}</t>
+          <t>{"assertions":["The creation header and form fill the available page content width.","The current create breadcrumb and section heading computed font sizes are 18px.","The current detail breadcrumb and detail information section heading computed font sizes are 18px.","No stepper or optional-upload control is rendered; one submit calls create once and does not call upload.","Switches are grouped within 12 pixels of their labels.","Paired controls use consistent label and field alignment."],"inputs":["desktop viewport","graph toggle","VLM toggle","paired model controls","valid create response"],"unit_boundary":"AIDP create form title, direct-submit flow, section layout and toggle grouping"}</t>
         </is>
       </c>
       <c r="Q17" s="5" t="inlineStr"/>
@@ -5702,8 +5708,10 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>AKPR-RULE-015
-AKPR-RULE-016</t>
+          <t>AKPR-RULE-010
+AKPR-RULE-015
+AKPR-RULE-016
+AKPR-RULE-017</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -5733,7 +5741,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Verify the rendered guide, knowledge cards, pagination, inline switches and paired create-form controls against the AIDP design at desktop and narrow widths.</t>
+          <t>Verify the rendered guide, knowledge cards, pagination, inline switches, title typography and direct create flow against the AIDP design at desktop and narrow widths.</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -5752,27 +5760,31 @@
         <is>
           <t>1. Open the overview and capture the expanded guide and first card row. =&gt; At desktop width each row contains four 148px-high cards with 16px horizontal gaps and 12px vertical gaps. Cards have 24px horizontal and 16px vertical padding, a 40px icon, a 16px/500/24px title, a full-width two-line 12px/20px description, and one 12px/18px metadata row. The toolbar search is 360px by 32px, the primary button is 32px high, and the selected view uses the primary blue background. Pagination is aligned right, uses 32px controls, puts page-size selection before page numbers, and has a pale-blue selected page with no primary border.
 2. Switch to table view and inspect the toolbar and column controls. =&gt; The create and view buttons align at the right, table column control follows them, and no edit operation appears in the overview. The table header and data rows are 40px high with 14px/22px body text and pale
-3. Open creation and inspect the page header, switches and paired fields at both viewport sizes. =&gt; The page uses the available width, switches sit beside their labels, and paired inputs or sliders align without page-level horizontal overflow.</t>
+3. Open creation and inspect the page title, section titles, switches and paired fields at both viewport sizes. =&gt; Breadcrumb labels and form section headings use 18px text, there is no step indicator or optional import stage, the page uses the available width, switches sit beside their labels, and paired inputs or sliders align without page-level horizontal overflow.
+4. Fill the required configuration and submit the create form. =&gt; The knowledge base is created directly with one create request, the browser opens its detail page, and no upload request is issued from creation.
+5. Open the detail page's information tab. =&gt; The detail breadcrumb and configuration, graph and permission section headings render at 18px.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
           <t>The running AIDP pages match the accepted layout and preserve Nexent visual conventions.
+The create and detail current page titles and detail information section headings use 18px text.
+The create flow has no stepper or optional upload stage; file upload remains in the knowledge base detail page.
 The expanded guide uses the pale-blue gradient introduction panel with 24px padding, a configuration-flow heading and three 156px-high step cards; the step content stays create, upload and configure an agent, and collapse or reopen preserves the overview state.
 The narrow viewport remains usable without overlapping labels or page-level horizontal scrolling.
 Collapsing the guide preserves the keyword and page; changing page size resets to page one; the last partial page keeps the same content-panel height; a valid page jump navigates without a mutating request.
-No write request is issued while visually inspecting the pages.</t>
+No write request is issued while inspecting pages before the explicit create submit.</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>No knowledge base is created, edited or deleted during this journey.
+          <t>No knowledge base is created before the explicit submit, edited, or deleted; the submit issues exactly one create request and no upload request.
 No global style or ES page behavior is changed.</t>
         </is>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>{"actor":"Authenticated AIDP tenant user","failure_evidence":["Save screenshots, computed layout measurements and browser console errors for both viewport sizes."],"final_business_result":["Users see the intended list and creation composition before beginning a knowledge-base operation."],"journey":["Inspect the overview guide and cards.","Inspect the table toolbar and pagination.","Inspect the full-page creation layout at desktop and narrow widths."]}</t>
+          <t>{"actor":"Authenticated AIDP tenant user","failure_evidence":["Save screenshots, computed layout measurements and browser console errors for both viewport sizes."],"final_business_result":["Users can inspect the intended list and create composition, then create a knowledge base directly and continue to its detail page."],"journey":["Inspect the overview guide and cards.","Inspect the table toolbar and pagination.","Inspect the full-page creation layout at desktop and narrow widths."]}</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(aidp): refine knowledge detail editing
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -630,7 +630,8 @@
 AKDT-RULE-005
 AKDT-RULE-006
 AKDT-RULE-007
-AKDT-RULE-008</t>
+AKDT-RULE-008
+AKDT-RULE-009</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -1058,12 +1059,13 @@
       <c r="D3" s="5" t="inlineStr">
         <is>
           <t>AKDT-RULE-001
-AKDT-RULE-007</t>
+AKDT-RULE-007
+AKDT-RULE-009</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Detail information reads graph configuration and group access without truthiness coercion</t>
+          <t>Detail information reads configuration and keeps edit controls scoped</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -1088,32 +1090,36 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Verify the detail page projects the returned configuration and local group permission while preserving false, zero and unknown values.</t>
+          <t>Verify the detail page projects returned configuration, preserves false and zero values, and keeps metadata, permission and Top K edits in their intended controls.</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Render a KB detail response with graph_config represented once as JSON text and once as an object.
-Include explicit false and zero values, private/shared permission variants and one missing safety value.</t>
+Include explicit false and zero values, private/shared permission variants and one missing safety value.
+Grant edit access and provide an available user-group option for the edit-control checks.</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>{"graph_config_forms":["json_string","object"],"profile":"mock"}</t>
+          <t>{"graph_config_forms":["json_string","object"],"profile":"mock","topk_range":[1,100]}</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
           <t>1. Render the configuration and graph sections for each response shape. =&gt; Values appear in their corresponding named fields and a model name is not duplicated.
 2. Inspect false, zero and missing values. =&gt; False and zero remain off/zero; a missing safety value is shown as unknown.
-3. Render private and shared permission records with group IDs. =&gt; Scope and group names follow local permission data and the viewer's group-read permission.</t>
+3. Render private and shared permission records with group IDs. =&gt; Scope and group names follow local permission data and the viewer's group-read permission.
+4. Open the header edit, lower permission edit and vector Top K edit. =&gt; The header form shows name, description and visible permission/group fields without a collapsed advanced section; the lower editor contains only permission and group fields; Top K uses the create-page slider and numeric value control.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>JSON text and object graph settings render consistently.
 Boolean false and numeric zero remain distinct from missing values.
-Effective permission and available group names come from the permission layer.</t>
+Effective permission and available group names come from the permission layer.
+The lower permission save sends only permission/group fields; the header form remains the only name/description editor.
+The Top K editor uses a 1-100 slider with a numeric value control.</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
@@ -1124,7 +1130,7 @@
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Graph fields and the two separate Top K values render under the correct labels.","Explicit false and zero are preserved while absent values remain unknown.","Group names render only with group:read permission."],"inputs":["AIDP detail payload","graph_config value","local group permission record"],"unit_boundary":"AIDP knowledge detail configuration parsing and permission presentation"}</t>
+          <t>{"assertions":["Graph fields and the two separate Top K values render under the correct labels.","Explicit false and zero are preserved while absent values remain unknown.","Group names render only with group:read permission.","Header and lower permission edit forms expose their separate allowed fields and omit the advanced-options collapse.","The vector Top K edit control matches the creation page slider layout and range."],"inputs":["AIDP detail payload","graph_config value","local group permission record","header and permission edit modes","vector Top K value"],"unit_boundary":"AIDP knowledge detail configuration, permission presentation and edit controls"}</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr"/>
@@ -5148,16 +5154,16 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>{"locale":"zh-CN","profile":"mock","status_values":[0,1,2,3,4,5],"task_retention_days":30}</t>
+          <t>{"locale":"zh-CN","profile":"mock","status_values":[0,1,2,3,4,5],"task_retention_days":30,"vector_topk_range":[1,100]}</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>1. Open the overview and click a card or knowledge-base name. =&gt; A full-width detail page opens with a breadcrumb, header and the three tabs Files, Upload tasks and Details; no list edit action remains.
+          <t>1. Open the overview and click a card or knowledge-base name. =&gt; A full-width detail page opens with a breadcrumb, header and the three tabs Files, Upload tasks and Details; no list edit action remains, and the console has no deprecated AIDP Modal or Drawer API warnings.
 2. Inspect Files and search by file name. =&gt; Only ingested files appear; download and delete follow the user's permission; pagination and table controls stay in the detail page.
 3. Open Upload tasks, search a name and choose each status filter. =&gt; The page states tasks are retained for 30 days, status values 0-5 are sent, statistics remain independent from the current page, and processing rows do not appear as ingested files.
 4. Open a failed task's failure details and retry it from the row action. =&gt; The drawer shows returned values only; retry submits a one-item file_uuids array and subsequent refresh reads the changed task status.
-5. Open Details and edit supported name/description, a supported setting and group permissions. =&gt; Each save sends only its own changed fields and updates the returned value; unsupported similarity edits are absent.</t>
+5. Open Details and edit metadata from the header, a supported setting, then permission and groups from the permission section. =&gt; Header edit shows name, description and directly visible permission/group controls; the lower editor contains only permission/group controls and sends no metadata fields; vector Top K uses the create-page slider style; unsupported similarity edits are absent.</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -5165,7 +5171,9 @@
           <t>The page has the exact three tabs and full content width.
 Ingested files and upload history remain separate live AIDP sources.
 Status filters, raw status rendering, failure details and single-file retry follow the contract.
-Detail settings and group permissions use separate authorized save operations.</t>
+Detail settings and group permissions use separate authorized save operations.
+The header edit is the only path that submits a changed name or description; the lower permission editor submits only permission and group values.
+The vector Top K editor uses the same slider and numeric value control as the creation form.</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -5760,7 +5768,7 @@
         <is>
           <t>1. Open the overview and capture the expanded guide and first card row. =&gt; At desktop width each row contains four 148px-high cards with 16px horizontal gaps and 12px vertical gaps. Cards have 24px horizontal and 16px vertical padding, a 40px icon, a 16px/500/24px title, a full-width two-line 12px/20px description, and one 12px/18px metadata row. The toolbar search is 360px by 32px, the primary button is 32px high, and the selected view uses the primary blue background. Pagination is aligned right, uses 32px controls, puts page-size selection before page numbers, and has a pale-blue selected page with no primary border.
 2. Switch to table view and inspect the toolbar and column controls. =&gt; The create and view buttons align at the right, table column control follows them, and no edit operation appears in the overview. The table header and data rows are 40px high with 14px/22px body text and pale
-3. Open creation and inspect the page title, section titles, switches and paired fields at both viewport sizes. =&gt; Breadcrumb labels and form section headings use 18px text, there is no step indicator or optional import stage, the page uses the available width, switches sit beside their labels, and paired inputs or sliders align without page-level horizontal overflow.
+3. Open creation and inspect the page title, section titles, switches and paired fields at both viewport sizes. =&gt; Breadcrumb labels and form section headings use 18px text, there is no step indicator or optional import stage, the page uses the available width, switches sit beside their labels, and paired inputs or sliders align without page-level horizontal overflow. The browser console has no deprecated Ant Design Modal, Drawer or Alert API warnings.
 4. Fill the required configuration and submit the create form. =&gt; The knowledge base is created directly with one create request, the browser opens its detail page, and no upload request is issued from creation.
 5. Open the detail page's information tab. =&gt; The detail breadcrumb and configuration, graph and permission section headings render at 18px.</t>
         </is>

</xml_diff>

<commit_message>
feat(aidp): upload selected files in a shared batch progress drawer
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_D2'!$A$1:$AA$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$8</definedName>
@@ -687,7 +687,8 @@
 AKPR-RULE-013
 AKPR-RULE-015
 AKPR-RULE-016
-AKPR-RULE-017</t>
+AKPR-RULE-017
+AKPR-RULE-018</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -763,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA21"/>
+  <dimension ref="A1:AA22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -784,9 +785,9 @@
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -2655,33 +2656,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>CMSR-D1-001</t>
+          <t>AKPR-D1-015</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>CMSR-005</t>
+          <t>AKPR-001</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>CMSR-005</t>
+          <t>AKPR-001</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>CMSR-RULE-013
-CMSR-RULE-014</t>
+          <t>AKPR-RULE-018</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Observer emits safe content before stream completion</t>
+          <t>AIDP import drawer uploads on selection and keeps results until confirmation</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>SDK-UT</t>
+          <t>FE-COMP</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2701,40 +2701,45 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Verify bounded marker lookahead and attempt state reset.</t>
+          <t>Verify selection immediately uploads valid files, actual transfer progress is distinct from AIDP acceptance, and Confirm closes without a second upload.</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Create an isolated observer and a controlled chunk sequence.</t>
+          <t>Render the import drawer with a writable mock knowledge base and a mocked upload API response.</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>{"profile":"mock","sequence":"failed partial, rollback, successful split code and think markers"}</t>
+          <t>{"file":"guide.txt","profile":"mock","upload_bytes":[716800,2621440]}</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>1. Feed a safe prefix and pause the source. =&gt; The prefix is emitted before flush or commit.
-2. Roll back the first attempt and feed split markers in the second. =&gt; The second output is ordered and contains no first-attempt residue.</t>
+          <t>1. Select multiple supported files together. =&gt; One multipart batch starts automatically; every row has a dashed gray border and Confirm is disabled while the request is active.
+2. Report intermediate progress, then complete browser transfer without resolving the upload response. =&gt; Each uploading ring shows the same batch percentage; the second line only shows the file size. Transfer completion changes rings to waiting indicators, borders stay dashed, Confirm remains disabled, and no delete action is present.
+3. Resolve the upload response as accepted. =&gt; The row changes to a solid near-black border and the accepted file id is passed to the parent refresh flow; the drawer remains open.
+4. Click Confirm. =&gt; The drawer closes and no additional upload request is sent.</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>The earliest safe content is observable before completion.
-Split markers retain their original semantics.</t>
+          <t>Choosing a valid file immediately uploads it through the existing AIDP route.
+Progress text and ring are derived from the upload event, not a timer.
+A successful response changes the row border to solid near-black.
+Results remain visible until Confirm, which never sends files again.</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>No stale fragment crosses attempts.
-No code is executed by the observer.</t>
+          <t>No per-file transferred-byte text or batch-progress label is rendered.
+No retry action is rendered in the import row.
+No change to the ES upload component.</t>
         </is>
       </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Safe prefix emitted before flush.","Raw code tag retained.","No failed-attempt residue."],"inputs":["normal content","split &lt;think&gt; and &lt;/think&gt;","raw &lt;code&gt; content"],"unit_boundary":"Observer.add_model_new_token and attempt lifecycle"}</t>
+          <t>{"assertions":["The upload API is called on selection and not on confirmation.","The rows share batch percentage rings and display only their own total file sizes while uploading.","Mixed responses map by file name; accepted rows become solid near-black and are reported to their parent. Only failed rows show delete; deleting removes a frontend row without any network call. Network errors mark all rows failed and enable Confirm. A 50-file selection makes one request, and further batches contain only newly selected files."],"inputs":["mock knowledge base","supported file","progress event","accepted upload response"],"unit_boundary":"AIDP import drawer automatic upload, progress, result retention and confirmation"}</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr"/>
@@ -2745,17 +2750,20 @@
       </c>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>pytest</t>
+          <t>vitest
+vitest</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>test/automation/d1/test_model_attempt_stream.py</t>
+          <t>test/automation/d1/AidpImportDrawer.test.tsx
+test/automation/d1/AidpUploadService.test.tsx</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>test_cmsr_d1_001</t>
+          <t>AKPR-D1-015
+AKPR-D1-015</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2772,85 +2780,214 @@
       </c>
       <c r="Z18" s="5" t="inlineStr">
         <is>
-          <t>sha256:625e8c8829b51b9cd91344555d05c5ebfdc7bd766d8485eab99b9f22773f3233</t>
+          <t>sha256:6c4a5f0c2060b7e3780c73a01331faeae9528c1f10de5bb60e37c8fcdfb54355</t>
         </is>
       </c>
       <c r="AA18" s="5" t="inlineStr">
         <is>
-          <t>sha256:242f1aaf8a5fe4427f503e5acb8db2cc6cb5096782c2e4fdf49fcb17ec471420</t>
+          <t>sha256:2bd0dcafdd0bd3669182569189845378bce21ae3c9ce22083b83b9fdca5ad631</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>CMSR-D1-001</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>CMSR-005</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>CMSR-005</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>CMSR-RULE-013
+CMSR-RULE-014</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Observer emits safe content before stream completion</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Verify bounded marker lookahead and attempt state reset.</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Create an isolated observer and a controlled chunk sequence.</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock","sequence":"failed partial, rollback, successful split code and think markers"}</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>1. Feed a safe prefix and pause the source. =&gt; The prefix is emitted before flush or commit.
+2. Roll back the first attempt and feed split markers in the second. =&gt; The second output is ordered and contains no first-attempt residue.</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>The earliest safe content is observable before completion.
+Split markers retain their original semantics.</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>No stale fragment crosses attempts.
+No code is executed by the observer.</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Safe prefix emitted before flush.","Raw code tag retained.","No failed-attempt residue."],"inputs":["normal content","split &lt;think&gt; and &lt;/think&gt;","raw &lt;code&gt; content"],"unit_boundary":"Observer.add_model_new_token and attempt lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr"/>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_model_attempt_stream.py</t>
+        </is>
+      </c>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>test_cmsr_d1_001</t>
+        </is>
+      </c>
+      <c r="V19" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W19" s="5" t="inlineStr"/>
+      <c r="X19" s="5" t="inlineStr"/>
+      <c r="Y19" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z19" s="5" t="inlineStr">
+        <is>
+          <t>sha256:625e8c8829b51b9cd91344555d05c5ebfdc7bd766d8485eab99b9f22773f3233</t>
+        </is>
+      </c>
+      <c r="AA19" s="5" t="inlineStr">
+        <is>
+          <t>sha256:242f1aaf8a5fe4427f503e5acb8db2cc6cb5096782c2e4fdf49fcb17ec471420</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
           <t>CMSR-D1-002</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-014
 CMSR-RULE-015</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Running step labels precede reasoning and survive retry rollback</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>FE-COMP</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Verify immediate running labels, rollback preservation, legacy history and removal of terminal label-only cards.</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Create the streaming adapter with a controlled SSE fixture.</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequences":["step 1, failed attempt, rollback, successful raw code, parse","legacy content before step label"]}</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>1. Emit a step label before any model content. =&gt; A running reasoning card displays Step 1 immediately.
 2. Roll back a partial attempt and stream successful raw code. =&gt; Step 1 remains during rollback and only successful raw code follows it.
 3. Parse and reload both new and legacy-order history. =&gt; One code card and one labeled nonempty reasoning card remain; a terminal label-only card is absent.</t>
         </is>
       </c>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>Step label appears before first token.
 Rollback preserves the label.
@@ -2858,326 +2995,326 @@
 Old history prepends late labels.</t>
         </is>
       </c>
-      <c r="O19" s="5" t="inlineStr">
+      <c r="O20" s="5" t="inlineStr">
         <is>
           <t>No failed-attempt content.
 No duplicate code card.
 No sibling invocation mutation.</t>
         </is>
       </c>
-      <c r="P19" s="5" t="inlineStr">
+      <c r="P20" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Running label is visible before content.","Terminal label-only step is hidden.","Successful code is visible after the label before commit.","History equals live output."],"inputs":["step_count","model_attempt_control","model_output_thinking","parse"],"unit_boundary":"Frontend live and history reasoning projection"}</t>
         </is>
       </c>
-      <c r="Q19" s="5" t="inlineStr"/>
-      <c r="R19" s="5" t="inlineStr">
+      <c r="Q20" s="5" t="inlineStr"/>
+      <c r="R20" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S19" s="5" t="inlineStr">
+      <c r="S20" s="5" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="T19" s="5" t="inlineStr">
+      <c r="T20" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_reasoning_card.ts</t>
         </is>
       </c>
-      <c r="U19" s="5" t="inlineStr">
+      <c r="U20" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-002</t>
         </is>
       </c>
-      <c r="V19" s="5" t="inlineStr">
+      <c r="V20" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W19" s="5" t="inlineStr"/>
-      <c r="X19" s="5" t="inlineStr"/>
-      <c r="Y19" s="5" t="inlineStr">
+      <c r="W20" s="5" t="inlineStr"/>
+      <c r="X20" s="5" t="inlineStr"/>
+      <c r="Y20" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z19" s="5" t="inlineStr">
+      <c r="Z20" s="5" t="inlineStr">
         <is>
           <t>sha256:b614502639e969ab0f3840d1381f1b12b01cb5b693a0b02d17387192b230b354</t>
         </is>
       </c>
-      <c r="AA19" s="5" t="inlineStr">
+      <c r="AA20" s="5" t="inlineStr">
         <is>
           <t>sha256:03f5fae5200c76ca296c75ab0ebf225f190fb3fe6a7f52c7c8c7e0da2a97d07c</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-003</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-014
 CMSR-RULE-016</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>CoreAgent commits streamed valid semantic repair</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>A protocol-invalid first attempt rolls back while its single preceding step label survives and the corrected result streams and commits.</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>A controlled model yields an invalid response then a pausable valid code action at step one.</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequence":"invalid code, rollback, corrected code chunks, commit, parse"}</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>1. Begin step one and return protocol-invalid model content. =&gt; Exactly one step label precedes begin; the attempt rolls back and one repair is scheduled.
 2. Pause the valid repair after its first safe chunk. =&gt; That chunk is visible before model completion.
 3. Complete the repair and classify it. =&gt; Its attempt commits and a single parse follows.</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>Corrected content is streamed and committed.
 Only the corrected action is executed.
 Lifecycle logs identify the repair without content.</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>No failed content after rollback.
 No repair instruction in user output.
 No suppressed successful stream.</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr">
+      <c r="P21" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Step label occurs before both model attempts and only once.","Successful repair does not set stream suppression.","Corrected attempt commits once.","Invalid attempt rolls back once."],"inputs":["step one","invalid model content","valid streamed &lt;code&gt; action"],"unit_boundary":"CoreAgent semantic repair and deferred model attempt lifecycle"}</t>
         </is>
       </c>
-      <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="5" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S20" s="5" t="inlineStr">
+      <c r="S21" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T20" s="5" t="inlineStr">
+      <c r="T21" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_semantic_repair_stream.py</t>
         </is>
       </c>
-      <c r="U20" s="5" t="inlineStr">
+      <c r="U21" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_003</t>
         </is>
       </c>
-      <c r="V20" s="5" t="inlineStr">
+      <c r="V21" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W20" s="5" t="inlineStr"/>
-      <c r="X20" s="5" t="inlineStr"/>
-      <c r="Y20" s="5" t="inlineStr">
+      <c r="W21" s="5" t="inlineStr"/>
+      <c r="X21" s="5" t="inlineStr"/>
+      <c r="Y21" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z20" s="5" t="inlineStr">
+      <c r="Z21" s="5" t="inlineStr">
         <is>
           <t>sha256:7ef8664f2224d068d7deafecf80f09353d734bc10b35a1147b3cc58d1ae6eacd</t>
         </is>
       </c>
-      <c r="AA20" s="5" t="inlineStr">
+      <c r="AA21" s="5" t="inlineStr">
         <is>
           <t>sha256:1dee7e7ce90f70c40d02907f11be7b55665495fdcaa3dfdec3ab478953c5c38c</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-004</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-018</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Rejected model output diagnostics distinguish budget exhaustion without default content leakage</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>Correlate each protocol rejection to the model response shape and budget while gating bounded raw previews.</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>Use isolated model diagnostics for a reasoning-only length response and a malformed nonempty response.</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L22" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","responses":["length with 4096 reasoning-only output tokens","malformed nonempty code Action"]}</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M22" s="5" t="inlineStr">
         <is>
           <t>1. Reject a reasoning-only length response with diagnostics disabled. =&gt; The log records model, attempt, requested and consumed tokens, reasoning and content counts, and reasoning-only budget exhaustion without raw text.
 2. Reject a malformed content response. =&gt; The distinct protocol reason and response shape are logged under its own attempt identifier.
 3. Enable diagnostic content preview for a rejected response longer than the preview cap. =&gt; Only a single escaped bounded prefix of model content and reasoning is logged; the full text remains absent.</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>Each rejection is attributable to one attempt and specific failure class.
 Raw output is absent by default and bounded on explicit opt-in.</t>
         </is>
       </c>
-      <c r="O21" s="5" t="inlineStr">
+      <c r="O22" s="5" t="inlineStr">
         <is>
           <t>No model output or user prompt enters SSE or persisted history from diagnostics.
 No secret or full raw payload is logged by default.
 No retry-budget or execution behavior changes.</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr">
+      <c r="P22" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Reasoning-only budget exhaustion flag is accurate.","Logs include attempt and token counts.","Default logs omit raw content.","Opt-in previews are escaped and capped."],"inputs":["finish_reason=length","reasoning_content","invalid code Action","explicit diagnostic flag"],"unit_boundary":"OpenAI model response diagnostics and CoreAgent protocol-error logging"}</t>
         </is>
       </c>
-      <c r="Q21" s="5" t="inlineStr"/>
-      <c r="R21" s="5" t="inlineStr">
+      <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S21" s="5" t="inlineStr">
+      <c r="S22" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T21" s="5" t="inlineStr">
+      <c r="T22" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_protocol_rejection_diagnostics.py</t>
         </is>
       </c>
-      <c r="U21" s="5" t="inlineStr">
+      <c r="U22" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_004</t>
         </is>
       </c>
-      <c r="V21" s="5" t="inlineStr">
+      <c r="V22" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W21" s="5" t="inlineStr"/>
-      <c r="X21" s="5" t="inlineStr"/>
-      <c r="Y21" s="5" t="inlineStr">
+      <c r="W22" s="5" t="inlineStr"/>
+      <c r="X22" s="5" t="inlineStr"/>
+      <c r="Y22" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z21" s="5" t="inlineStr">
+      <c r="Z22" s="5" t="inlineStr">
         <is>
           <t>sha256:9f06a6565fff8e542fdcb89725b5fc7f669ad52b07301bdc99aa3e2eba23552c</t>
         </is>
       </c>
-      <c r="AA21" s="5" t="inlineStr">
+      <c r="AA22" s="5" t="inlineStr">
         <is>
           <t>sha256:a53056127d5f2efce4a9d98c92c9c97892451de0d1d353603584612c0a9ef1ba</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA21"/>
+  <autoFilter ref="A1:AA22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5407,15 +5544,18 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>1. Open the writable knowledge base and upload a document. =&gt; The document appears and its processing status reaches a terminal state through polling.
-2. Download the processed document. =&gt; The browser receives the original file with its name.
-3. Delete the document and confirm the dialog. =&gt; The document disappears from the list and the deletion reports its own result.
-4. Open the read-only knowledge base and attempt the same operations. =&gt; Upload and delete are unavailable while browsing and download remain permitted.</t>
+          <t>1. Open the writable knowledge base and choose Import files. =&gt; A 764px right-side drawer opens with the click-or-drop area, supported-format notes, a scrollable file list and fixed Cancel/Confirm actions.
+2. Select or drop a supported document, wait for the upload response and then activate Confirm. =&gt; Selection starts upload immediately; transfer completion shows waiting until AIDP responds. Accepted rows become solid near-black and remain visible; Confirm closes without uploading again.
+3. Wait for the accepted document's processing status to reach a terminal state. =&gt; The document appears and its processing status reaches a terminal state through polling.
+4. Download the processed document. =&gt; The browser receives the original file with its name.
+5. Delete the document and confirm the dialog. =&gt; The document disappears from the list and the deletion reports its own result.
+6. Open the read-only knowledge base and attempt the same operations. =&gt; Upload and delete are unavailable while browsing and download remain permitted.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Upload reaches a terminal processing state.
+The import drawer keeps completed and failed rows visible, with independent scrolling and fixed Confirm action; it exposes no retry action.
 The downloaded file matches the uploaded original.
 Deletion removes the document after confirmation.
 Permission gates match the documented read and edit rules.</t>
@@ -5430,7 +5570,7 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>{"actor":"Authenticated test tenant user","failure_evidence":["Retain browser screenshot, network log, downloaded file metadata and console trace on failure."],"final_business_result":["A user with edit permission can add, retrieve and remove documents while a read-only user can only browse and download them."],"journey":["Open a writable knowledge base file view.","Upload and wait for processing to finish.","Download the document.","Delete the document with confirmation.","Check the same controls on a read-only base."]}</t>
+          <t>{"actor":"Authenticated test tenant user","failure_evidence":["Retain browser screenshot, network log, downloaded file metadata and console trace on failure."],"final_business_result":["A user with edit permission can add, retrieve and remove documents while a read-only user can only browse and download them."],"journey":["Open a writable knowledge base file view and its import drawer.","Select a supported document, observe its automatic upload, confirm the drawer and wait for processing to finish.","Download the document.","Delete the document with confirmation.","Check the same controls on a read-only base."]}</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">

</xml_diff>

<commit_message>
fix(aidp): align knowledge creation with live API contract
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -2164,43 +2164,43 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Verify graph configuration serialization, the inverse thinking mapping, the independent Top K values and the prompt byte limit.</t>
+          <t>Verify live graph configuration serialization, the inverse Chinese thinking mapping, absence of graph Top K and the 1 to 4096 character prompt limit.</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Prepare graph payloads with the switch on and off, both languages and prompt lengths around the byte limit.</t>
+          <t>Prepare graph payloads with the switch on and off, both languages and Unicode prompt lengths around the character limit.</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>{"domains":["general","medical"],"languages":["chinese","english"],"profile":"mock","prompt_bytes":[2048,2049]}</t>
+          <t>{"domains":["常规","医疗","法律法规"],"languages":["中文","英文"],"profile":"mock","prompt_characters":[0,1,4096,4097]}</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>1. Submit a graph configuration with the thinking switch enabled. =&gt; The thinking mode field is false and the graph keys use their documented names.
-2. Submit a knowledge base Top K together with a graph Top K. =&gt; The two values are serialized independently without overwriting each other.
-3. Submit prompts at and beyond the byte boundary together with a disabled graph. =&gt; The limit passes at the boundary, longer input is rejected and a disabled graph omits its configuration entirely.</t>
+          <t>1. Submit a graph configuration with the thinking switch enabled. =&gt; The no_think_mode field is the Chinese string 否 and only the seven template keys plus llm_model_name are forwarded.
+2. Submit a knowledge base Top K with an obsolete graph Top K key. =&gt; The outer topk is preserved and the obsolete graph key is not forwarded.
+3. Submit prompts at and beyond the character boundary together with a disabled graph. =&gt; The limit passes at the boundary, longer input is rejected and a disabled graph omits its configuration entirely.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
           <t>The thinking switch maps inversely onto the thinking mode field.
-Both Top K values survive independently.
-The prompt limit is enforced in UTF-8 bytes.</t>
+Only the outer knowledge-base topk is submitted.
+The prompt limit is enforced as 1 to 4096 Unicode characters.</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
           <t>No hidden previous graph configuration is submitted when the graph is off.
-No graph Top K overwrites the knowledge base Top K.
+No graph Top K key reaches AIDP.
 No invented JSON key names.</t>
         </is>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["The thinking mode field is false when thinking is enabled.","Graph and knowledge base Top K stay independent.","Prompt length is measured in UTF-8 bytes.","Disabled graph omits its configuration."],"inputs":["graph switch","domain","graph top k","hop count","thinking switch","prompt language","prompt text"],"unit_boundary":"Graph configuration validation and serialization"}</t>
+          <t>{"assertions":["The thinking mode field is 否 when thinking is enabled.","Only outer knowledge-base topk survives.","Prompt length is measured in Unicode characters.","Disabled graph omits its configuration."],"inputs":["graph switch","domain","obsolete graph top k","hop count","thinking switch","prompt language","prompt text"],"unit_boundary":"Graph configuration validation and serialization"}</t>
         </is>
       </c>
       <c r="Q13" s="5" t="inlineStr"/>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Graph and multimodal models are queried from separate categories with independent caches</t>
+          <t>One model query populates three categories and graph templates preserve edited prompts</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -2271,12 +2271,12 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Verify the model category split, the independent query caches and the omission of hidden model values.</t>
+          <t>Verify one model query, category separation by model_type, label and identifier mapping, hidden value omission and graph template interaction.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Render the creation form with stubbed model queries per category and both capability switches toggled.</t>
+          <t>Render the creation form with one model response, graph templates in both languages and both capability switches toggled.</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -2286,49 +2286,76 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>1. Enable the graph section. =&gt; The graph model query uses the llm category and fills the graph model field.
-2. Enable multimodal captioning. =&gt; The multimodal model query uses the vlm category and fills the multimodal field independently.
+          <t>1. Enable the graph section. =&gt; One all-category query fills separate embedding, llm and vlm controls by model_type; graph activation reads the template endpoint.
+2. Enable multimodal captioning. =&gt; The multimodal field uses the vlm entries from the existing model result without another request.
 3. Disable each capability after a selection. =&gt; The hidden model value is absent from the submitted payload.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>Each model field is populated from its own category.
-Caches and selections never mix.
+          <t>Each field is populated from its model_type, displays display_name and submits model_name.
+A shared model cache never mixes category selections. Domain and language changes preserve manual prompts, and restore uses the current template. Template failures block graph-enabled creation.
 Disabled capabilities submit no model value.</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>No llm result used for the multimodal field.
+          <t>No llm result used for the multimodal or embedding field.
 No hidden previous model resubmitted.
 No unverified model name silently defaulted.</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Graph query uses llm and multimodal uses vlm.","Caches are keyed independently.","Disabled capability clears its submitted model."],"inputs":["graph switch","multimodal switch","selected models","query cache keys"],"unit_boundary":"Creation form model queries, caches and hidden value handling"}</t>
+          <t>{"assertions":["One query returns all categories and controls filter by model_type.","Model data uses one shared query cache; templates are cached by language.","Disabled capability clears its submitted model."],"inputs":["graph switch","multimodal switch","selected models","query cache keys"],"unit_boundary":"Creation form model queries, caches and hidden value handling"}</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr"/>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>unbound</t>
-        </is>
-      </c>
-      <c r="S14" s="5" t="inlineStr"/>
-      <c r="T14" s="5" t="inlineStr"/>
-      <c r="U14" s="5" t="inlineStr"/>
-      <c r="V14" s="5" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>vitest
+vitest</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/AidpCreateKbPage.test.tsx
+test/automation/d1/AidpCreateKbSections.test.tsx</t>
+        </is>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>AKPR-D1-011
+AKPR-D1-011</t>
+        </is>
+      </c>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
       <c r="W14" s="5" t="inlineStr"/>
       <c r="X14" s="5" t="inlineStr"/>
       <c r="Y14" s="5" t="inlineStr">
         <is>
-          <t>未绑定</t>
-        </is>
-      </c>
-      <c r="Z14" s="5" t="inlineStr"/>
-      <c r="AA14" s="5" t="inlineStr"/>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z14" s="5" t="inlineStr">
+        <is>
+          <t>sha256:f2872957a3d2f7e49abdaf84e15a0bb4b0ac6bc46b8d5116ac7c58ced7988633</t>
+        </is>
+      </c>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>sha256:0074537ecfe51f517f3d749371770d0d8b5e1f7a3b96bef2a13e16f63fc18cbd</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2775,7 +2802,7 @@
       <c r="X18" s="5" t="inlineStr"/>
       <c r="Y18" s="5" t="inlineStr">
         <is>
-          <t>校验通过</t>
+          <t>实现哈希失效</t>
         </is>
       </c>
       <c r="Z18" s="5" t="inlineStr">
@@ -3978,7 +4005,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Verify the create proxy forwards chunking, retrieval, graph, model and safety fields while preserving legacy field names and existing defaults.</t>
+          <t>Verify the create proxy forwards the verified chunking, retrieval and model fields and graph JSON string, omits obsolete graph Top K and smartsplit, and preserves existing product defaults.</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -4161,7 +4188,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Model queries select a single category per control</t>
+          <t>Model query returns all advertised types when no service filter is supplied</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -4186,12 +4213,12 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Verify the model query proxy passes one category per request and returns only models applicable to the knowledge base application.</t>
+          <t>Verify the model query proxy omits the service filter for the unified query and returns models applicable to KnowledgeBase with their types, display names and identifiers.</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>A controllable upstream model fixture serves distinct payloads per category.</t>
+          <t>A controllable upstream model fixture serves an all-category payload and optional category-filtered responses.</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
@@ -4201,28 +4228,28 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>1. Query the graph model list. =&gt; The request carries the llm category and the response exposes only llm models.
-2. Query the multimodal model list. =&gt; The request carries the vlm category and the response exposes only vlm models.
+          <t>1. Query all models without a service parameter. =&gt; The request has app=KnowledgeBase without service and exposes embedding, llm and vlm models with model_type.
+2. Query models with an explicit vlm service filter. =&gt; The request carries the vlm category and the response exposes only vlm models.
 3. Query an unsupported or failing category. =&gt; A stable error or an empty result is returned without falling back to another category.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>One category is requested per control.
-Responses are not reused across categories.
+          <t>One query populates all three controls.
+Controls split the returned model types without changing identifiers.
 Failures do not silently substitute another category.</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>No shared cache entry across categories.
+          <t>No model_type category mixing.
 No fabricated model identifier on failure.
 No change to existing non-AIDP model endpoints.</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>{"endpoint":"/aidp-mgmt/models","method":"GET","protocol":"HTTP","request_expectations":["The service parameter carries exactly one requested category.","The application parameter keeps the knowledge base scope.","No credential is returned to the browser."],"response_expectations":["Only models of the requested category are returned.","An unavailable category yields a stable error or an empty list.","Results are filtered to the knowledge base application scope."]}</t>
+          <t>{"endpoint":"/aidp-mgmt/models","method":"GET","protocol":"HTTP","request_expectations":["The service parameter is optional; omitting it retrieves all categories.","The application parameter keeps the knowledge base scope.","No credential is returned to the browser."],"response_expectations":["Model response preserves model_type, model_name and display_name for applicable models.","An unavailable category yields a stable error or an empty list.","Results are filtered to the knowledge base application scope."]}</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(frontend): agent config high-fidelity layout, resource drawers and debug page
- High-fidelity agent config layout with selected resource rows and add button
- Resource picker drawers for models, skills, tools and child agents
- Agent creation guide and first-creation welcome experience
- High-fidelity debug layout with welcome and question suggestions
- configurationLayout/debugLayout support in Thread and Composer
- Tags mapping in published agent list service
- D1/D4 test assets, automation cases and handoff docs
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_D5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_D2'!$A$1:$AA$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_D5'!$A$1:$AA$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -551,11 +551,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -603,25 +603,153 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>High-fidelity Agent configuration layout</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Present an existing empty Agent draft using the measured four-card editor, actionable resource entries, and a five-question addition limit while preserving existing configuration and workflow contracts.</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-001
+AGENT-CONFIG-RULE-002
+AGENT-CONFIG-RULE-003
+AGENT-CONFIG-RULE-004
+AGENT-CONFIG-RULE-005
+AGENT-CONFIG-RULE-006
+AGENT-CONFIG-RULE-007
+AGENT-CONFIG-RULE-008
+AGENT-CONFIG-RULE-009
+AGENT-CONFIG-RULE-010
+AGENT-CONFIG-RULE-011</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>D1
+D4</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>{"notes":"The2026-10-08 partial handoff is historical. Current geometry comes from the2026-10-09 inspector handoff and user authorization. The2026-10-10 selected-tools/child-Agent bug directly extends this baseline; shell geometry reuses measured knowledge rows, while descendant values are frozen screenshot-based choices rather than new inspector claims. D1 proves component contracts; D4 proves browser geometry/scroll/workflow. D2,D3,D5 are excluded with boundary reasons in the formal design; no exact font or artwork parity is claimed without matching assets.","requirement_ids":["AGENT-CONFIG-REQ-001","AGENT-CONFIG-REQ-002","AGENT-CONFIG-REQ-003"],"spec_path":"../nexent-doc/docs/Developing/agt-editor-empty-configuration-layout/proposal.md"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CREATION-GUIDE</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Agent first-creation guide</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Explain four measured configuration workflow regions after new Agent creation.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-RULE-001
+AGENT-GUIDE-RULE-002
+AGENT-GUIDE-RULE-003</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>D1
+D4</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>{"notes":"Same-page inspector analysis precedes code. D2/D3/D5 excluded for unchanged protocol/provider/deployment. Browser preference has no server synchronization; proprietary font glyph parity unverified.","requirement_ids":["AGENT-GUIDE-REQ-001"],"spec_path":"../nexent-doc/docs/Developing/agt-editor-first-creation-guide/proposal.md"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Measured Agent debug panel</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Present draft debug below the shared editor identity row with measured welcome, single-column questions and composer while preserving chat controls.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-RULE-001
+AGENT-DEBUG-RULE-002
+AGENT-DEBUG-RULE-003</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>D1
+D4</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>{"notes":"Inspector numeric values are frozen in product handoff. D2/D3/D5 excluded for unchanged protocol/provider/deployment. Font glyph parity and unexposed gradient positions are unverified.","requirement_ids":["AGENT-DEBUG-REQ-001"],"spec_path":"../nexent-doc/docs/Developing/agt-editor-debug-panel-layout/proposal.md"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
           <t>AGENT-LIST-VIEWS</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Agent list grid and table views</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Switch between the existing agent cards and a data-backed table without changing page-level content or agent operations.</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-RULE-001
 AGENT-LIST-RULE-002
@@ -630,40 +758,40 @@
 AGENT-LIST-RULE-005</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>D1
 D4</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>{"notes":"User request and same-page WeMeeting high-fidelity reference; no Edge window inspected.","requirement_ids":["AGENT-LIST-REQ-001","AGENT-LIST-REQ-002"],"spec_path":"docs/handoffs/2026-10-08-agent-list-high-fidelity.md"}</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Silent model retry stream visibility</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Successful model attempts stream raw content while failed attempts leave no visible or persisted fragments.</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-013
 CMSR-RULE-014
@@ -673,7 +801,7 @@
 CMSR-RULE-018</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>D1
 D2
@@ -682,14 +810,14 @@
 D5</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>{"requirement_ids":["CMSR-005"],"spec_path":"nexent-doc/docs/Developing/chat-message-model-silent-retry/proposal.md"}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -700,12 +828,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -719,11 +847,11 @@
     <col width="42" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -872,21 +1000,996 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>AGENT-CONFIG-D1-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-REQ-001
+AGENT-CONFIG-REQ-002</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-001
+AGENT-CONFIG-RULE-002
+AGENT-CONFIG-RULE-003
+AGENT-CONFIG-RULE-004
+AGENT-CONFIG-RULE-005</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Regroup the empty draft into four cards without breaking section focus or action gates</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Verify four-card composition, preserved section state/focus, guardrail reachability, action validation/permission gates, and absence of writes from render/collapse using the AgentConfig component boundary.</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Render AgentConfig with an initialized Agent draft and mocked existing section components.
+Control mocked save outcomes and read-only state; expose localized keys as visible text.</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>{"card_count":4,"draft":{"asset_ref":"empty_agent_draft"},"profile":"mock","resource_order":["knowledge_base","conversation_guide","skills","tools","collaborative_agents"]}</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>1. Render AgentConfig with an initialized Agent draft. =&gt; Basic, model/prompt, shared-resource, and permission/advanced cards appear in one scroll region; all existing field groups including guardrail remain reachable, resources follow the design order, outer category tabs are absent, and workflow actions remain outside that region.
+2. Collapse a collapsible resource section, then issue matching NL2Agent resource and nested prompt focus requests. =&gt; The requested section reopens and scrolls into view, nested prompt targeting remains supported, and each request clears without losing draft values.
+3. Invoke unlock, debug, and publish actions. =&gt; Unlock and debug call their existing callbacks; publish validates and awaits save before opening the existing modal.
+4. Repeat debug/publish with rejected validation, failed save, and a read-only draft. =&gt; Failed validation/save prevents downstream actions; read-only disables editing/publication, while existing allowed read-only inspection remains reachable.</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>Exactly four outer card groups exist in one scroll region, including all existing field groups and guardrail.
+Shared resources follow knowledge/welcome/skills/tools/child-Agent order and start expanded.
+Section collapse and NL2Agent focus preserve draft values, reopen and scroll to the exact target.
+Successful actions retain callbacks; invalid or unsaved drafts do not invoke downstream debug/publication.
+Rendering, collapsing and focusing do not request backend updates; read-only prevents mutation/publication.</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Do not omit or duplicate any existing configuration section.
+Do not invoke backend services or mutate persisted Agent data as a result of rendering or collapsing sections.
+Do not bypass save/validation/permission checks or move workflow actions into the scrolling module list.</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Exactly four outer cards group existing field components; no outer category tabs appear.","Resources are in the specified order and guardrail remains available.","Collapse/focus reopens the targeted resource without dropping state and calls scrollIntoView.","Unlock/debug callbacks and publish modal occur only after applicable successful validation/save/permission gates.","Render/collapse/focus do not persist changes."],"inputs":["initialized Agent draft","localized strings","focus request","section interactions","action callbacks","save failure","read-only state"],"unit_boundary":"AgentConfig React component rendered inside Ant Design App and Form providers, with existing section components, Agent store, route query, translations, and save guard mocked."}</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>vitest
+vitest</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-config-layout.test.tsx
+test/automation/d1/agent-config-prompt.test.tsx</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-001
+AGENT-CONFIG-D1-001</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr"/>
+      <c r="X2" s="5" t="inlineStr"/>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>sha256:1b1b2c4ca225df799d587e0fd3d3d8c8104d29fe6a848848a6eda91cf3a9e1b4</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>sha256:ea731f17afcbdf014ef62b5400aa16c1b3dca7d2002b2304d8c1b1d8c6fbe117</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-002</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-REQ-002</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-005
+AGENT-CONFIG-RULE-007</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Limit new preset questions to five without truncating legacy drafts</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Execute the real AgentGuide component against controlled draft state to prove five-item additions, value-preserving edits/removal, and legacy six-item load compatibility.</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Render the real AgentGuide inside Ant Design Form/App with a mocked Agent store update callback and translations.
+Provide separate logical drafts with zero, four, five, and six stored questions.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"legacy_draft":{"asset_ref":"agent_draft_six_questions"},"question_counts":[0,4,5,6]}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Render zero questions and add one; edit its value and the greeting. =&gt; The localized counter uses maximum five and update callbacks retain the entered question/greeting values.
+2. Render four questions and add the fifth, then render the updated five-question state. =&gt; The callback appends exactly one empty question and add becomes disabled at5/5.
+3. Remove one of five questions and render the four-question result. =&gt; The correct item is removed, other values remain intact, and add re-enables.
+4. Render a legacy six-question draft without interacting. =&gt; All six question values remain rendered, add is disabled, and no update callback occurs from load.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>The effective maximum for additions and localized count/tooltip is five.
+Add is enabled below five and disabled at five or above.
+Greeting/question edits and removal retain the existing update contract and unaffected values.
+Legacy six-item drafts are not truncated or automatically saved.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>Do not discard legacy questions, make a write during render, or introduce a backend schema/API change.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["The fifth addition appends one item and the add control disables at the boundary.","Removal from five retains the other values and permits a new addition.","Six question values render unchanged without a load-time update.","Counter translation receives maximum5 and edits preserve expected payload values."],"inputs":["zero-question draft","four-question draft","five-question draft","legacy six-question draft","edit and remove interactions"],"unit_boundary":"Real AgentGuide component with controlled Agent-store state; UI behavior is not replaced by a mocked child."}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>vitest</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-config-guide.test.tsx</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-002</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:39a5d953b19d09f70343d9924881bd86e99d9753b149df34d69f60674f48b59a</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:4eb7abaf1a8199a4b3e5675079e93b771d0dc6ad9987f71f20d46c0444811b04</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-REQ-002</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-001
+AGENT-CONFIG-RULE-005
+AGENT-CONFIG-RULE-008
+AGENT-CONFIG-RULE-011</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Render ordered selected tool and child-Agent rows with actionable resource entries and preserved configuration/removal</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Execute the real resource-add control, ToolManagement and CollaborativeAgent to prove empty-entry compatibility, ordered compact selected rows, real metadata, configuration/removal callbacks and read-only behavior without render-time writes.</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Render the actual new or existing resource-add presentation with empty resources and explicit association/create callbacks.
+Mock existing resource services/state without replacing the add control or owning resource component.
+Render real populated ToolManagement and CollaborativeAgent in high-fidelity mode with logical catalog, saved child-version, internal/external relation and read-only fixtures; keep store/service hooks controlled.</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>{"association_count":0,"entry_height":48,"grid_gap":8,"reference_entry_width":602.5,"reference_row_width":1213,"selected_child_agents":{"asset_ref":"selected_internal_external_agents_with_saved_versions"},"selected_row":{"action_glyph_size":14,"action_target_size":24,"border_color":"#DFDFDF","child_avatar_size":32,"content_gap":8,"height":48,"horizontal_padding":12,"name_color":"#191919","name_font_size":14,"name_font_weight":400,"name_line_height":22,"radius":4,"tag_color":"#777777","tag_font_size":12,"tag_line_height":18,"tool_icon_size":24,"vertical_padding":8},"selected_tools":{"asset_ref":"selected_tools_with_managed_knowledge_tool"}}</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>1. Render the empty resource module without interacting. =&gt; A two-column row contains a first-column add entry with48px height, radius8, padding8/12 and3%
+2. Activate the add entry. =&gt; The association-selection path opens exactly once, with creation/manage callback untouched.
+3. Activate the separate new/manage action. =&gt; The creation/management path opens with association callback untouched.
+4. Repeat with a read-only resource module. =&gt; Mutation actions are disabled and do not invoke association/create callbacks.
+5. Render populated tool and child-Agent modules, including missing optional labels, a managed knowledge tool and a saved child version differing from the latest catalog version. =&gt; Visible resources keep their selection order in a two-column grid; names and real neutral tags share compact48px rows, full names and saved child versions remain available in tooltips, the add entry follows selected rows, managed knowledge tools remain hidden without removal from state, and rendering makes no mutation or relation request.
+6. Open settings on a configurable selected tool, remove one selected tool, then remove an internal and an external child Agent through their existing actions. =&gt; Tool configuration retains canonical parameters and prerequisites; tool removal preserves other tools including managed knowledge tools; internal removal updates matching ID/relation entries without changing other snapshots; external removal uses the existing relation-service callback and only updates selection on its successful result.
+7. Render populated read-only and default-mode modules and attempt disabled selected-row actions. =&gt; Read-only tool settings/removal and child removal do not mutate state; default mode retains its grouped tool and internal/external child presentation, and missing optional catalog labels produce no invented tag values.</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>Add remains in the left column and does not become a full-width dashed placeholder.
+Measured48px height,8px gap/radius and3% background are represented by the actual control.
+Association and creation callbacks are separate and permission gated.
+Real selected tool and child-Agent rows use the frozen common shell, names/tags, icon/avatar sizes and always-visible24px action targets, followed by the add entry.
+Real labels, full names and saved child versions remain available without invented screenshot data; managed knowledge tools stay in state but are not displayed.
+Configuration and internal/external removals retain existing callbacks, unaffected selections and read-only gates; default presentation remains compatible.</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>Do not persist a resource, duplicate associations, or call a creation API merely by rendering or opening selection.
+Do not remove managed knowledge tools, overwrite retained child versions, fabricate optional metadata, or restyle knowledge rows/association drawers.</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Two-column layout and first-column add entry retain measured styling.","Add and create interactions each call only their own workflow.","Render and disabled controls issue no mutation callback.","Selected rows represent the frozen shell/name/tag/icon/action contract and preserve selected order with the add entry last.","Settings opens the actual existing tool configuration path; removals change only intended selections/relations and preserve managed knowledge tools and other snapshots.","Read-only prevents selected-row mutations; missing optional metadata stays absent; saved-version/full-name tooltips and default presentation remain available."],"inputs":["empty resources","association callback","creation callback","read-only state","ordered populated tool and child-Agent selections","managed knowledge tool","canonical tool parameters and missing optional labels","saved child version and internal/external removal results","default presentation mode"],"unit_boundary":"Actual resource-add control, ToolManagement and CollaborativeAgent rendered with Ant Design providers and existing query/store/service hooks controlled; selected-row components and actions are not replaced by mocks."}</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>vitest
+vitest
+vitest</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-config-resources.test.tsx
+test/automation/d1/agent-config-selected-tools.test.tsx
+test/automation/d1/agent-config-selected-child-agents.test.tsx</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-003
+AGENT-CONFIG-D1-003
+AGENT-CONFIG-D1-003</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" s="5" t="inlineStr"/>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>sha256:402c8dfd7414a39feca412292b5eb1208615c0ff7c20bb1ac19bea4518e02ff9</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>sha256:3f76518606adc1486ff89c288c6cc27973bef01d7f4cbb2b0e8b6f9d50a7a53a</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-004</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-REQ-002</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-005
+AGENT-CONFIG-RULE-009</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Enforce measured text-entry limits without truncating stored drafts</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Exercise real AgentInfo, AgentGuide, and AgentPrompt inputs to verify measured high-fidelity limits, exact boundary entry, preserved legacy overlong values, and default-mode compatibility.</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Render real field components with Ant Design providers and controlled Agent-store callbacks.
+Provide separate empty, exact-boundary, and overlong legacy values without replacing the inputs with mocks.</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>{"description_limit":200,"duty_limit":1000,"greeting_limit":200,"legacy_description_length":201,"legacy_duty_length":1001,"legacy_greeting_length":201}</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>1. Render high-fidelity inputs and enter exactly 200 description/greeting characters and 1000 duty characters. =&gt; Entry limits expose the measured boundaries and existing callbacks retain complete boundary values.
+2. Render legacy overlong stored values without interaction, then shorten them below their measured limits. =&gt; Complete stored values remain visible without a load-time update; shortening produces the exact reduced value through the existing callback.
+3. Render default component mode with its preexisting field limits. =&gt; Default limits and legacy editing behavior remain compatible; the new high-fidelity limit is not applied globally.</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>High-fidelity description and greeting entry use a 200-character limit; duty uses 1000.
+Exact boundary values remain complete, and legacy overlong values are never sliced or silently persisted on load.
+Shortening stored overlong content remains possible and preserves expected callback payloads.
+Default-mode field constraints remain unchanged.</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>Do not truncate persisted content, write on render, or change backend request/response contracts.</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Actual input limits match 200, 200, and 1000 in high-fidelity mode.","Callback values preserve the full exact-boundary or shortened text.","Legacy values render intact without automatic callbacks.","Default-mode limits match the existing component contract."],"inputs":["empty values","boundary text","overlong legacy values","shortened text","default component mode"],"unit_boundary":"Real AgentInfo, AgentGuide, and AgentPrompt controls with store/query/resource dependencies controlled at their existing hook boundaries."}</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>vitest
+vitest
+vitest</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-config-info.test.tsx
+test/automation/d1/agent-config-guide.test.tsx
+test/automation/d1/agent-config-prompt.test.tsx</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-004
+AGENT-CONFIG-D1-004
+AGENT-CONFIG-D1-004</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr"/>
+      <c r="X5" s="5" t="inlineStr"/>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z5" s="5" t="inlineStr">
+        <is>
+          <t>sha256:5f33024788d9fdd9d967a2964c21b46f11e124a70f694e2afa90ec680e795aa4</t>
+        </is>
+      </c>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>sha256:7e2095b8a8c40bf6eda6b16139471fe337fedecbb0d4cc3824f9eaf86f2cdd13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-REQ-003</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-010</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Reuse the resource drawer and preserve controlled model membership and order</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Verify actual common drawer controls, scroll/mask, controlled model add/remove and no render-time selection callback.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Render real AddResourceDrawer and AddModelDrawer with existing model query controlled at its hook boundary.</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>{"model_ids":[2,1],"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>1. Open shared drawer and inspect right placement,mask,header and close/confirm controls. =&gt; Existing shared drawer design renders; close and confirm invoke only their supplied callbacks.
+2. Render model drawer with ordered configured IDs, remove a configured model and select a new model. =&gt; Callbacks retain remaining order and append new IDs without replacing priority or mutating on render.</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Shared right drawer is reused with original close/confirm callbacks.
+Controlled model add/remove preserves order and no callback occurs on render.
+Standalone drawer defaults remain compatible.</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Do not save on render/open/close or discard retained model IDs/overrides.</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Right masked drawer and scroll region render.","Model callbacks preserve remaining IDs and append newly selected ID.","Rendering does not change selection."],"inputs":["ordered model IDs","catalog","close/confirm interactions"],"unit_boundary":"Real shared drawer and model selector components with model query mocked."}</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>vitest</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-config-drawers.test.tsx</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D1-005</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:24f0b216ba67e0b9afc79033ba7c9a5d9ef8e4e816372d7826ec2ce091d460ce</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:e21f3380f462f54d1161a964b9ad41a485e43eda860cd66a055c6027889cda87</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-D1-001</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-REQ-001</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-RULE-002
+AGENT-DEBUG-RULE-003</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Draft welcome and preset selection preserve data and only fill composer</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Verify real debug welcome/questions with changing draft values, empty values and legacy arrays without request or configuration writes.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Render real welcome and suggestions with a controlled composer callback and logical draft data.</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>{"draft":{"asset_ref":"debug_agent_draft"},"profile":"mock","question_count":6}</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>1. Render name and greeting plus six stored questions. =&gt; Draft name/greeting and all six questions appear without truncation or source mutation.
+2. Select one question, then rerender with changed name/greeting and no questions. =&gt; Exact text is supplied once to the composer callback only; changed draft values replace prior text and empty questions omit the suggestion section.</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Dynamic values render exactly; selection calls composer only; empty and legacy values are preserved.</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>No HTTP/provider invocation
+no Agent update or automatic question send.</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["All six stored questions render; callback receives selected text once; no source data mutation; empty section omitted; rerender updates draft text."],"inputs":["draft name","greeting","six questions","changed values","empty questions","selection callback"],"unit_boundary":"Real debug welcome and suggestion React components with controlled selection callback"}</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>vitest</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-debug-layout.test.tsx</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-D1-001</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" s="5" t="inlineStr"/>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:fcc7927d11dea62a1dca00601a71032de78c6c3e21b4892668141efe56716e55</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:8ad5aeaa20600915a969d2c6f9fdf9c8a2415d87618086a9ddff3aad2115208c</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-D1-001</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CREATION-GUIDE</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-REQ-001</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-RULE-002
+AGENT-GUIDE-RULE-003</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Guide eligibility and completion remain scoped explanatory state</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>FE-COMP</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Prove creation-only eligibility, identity isolation, denied-storage fallback and navigation/dismissal without business effects.</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Render real guide with controlled identity/draft readiness and deterministic Tour boundary; use isolated browser storage.</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>{"draft":{"asset_ref":"newly_created_agent"},"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>1. Render creation entry and change loading/read-only/identity/completed conditions. =&gt; Only ready editable uncompleted creation context opens; ordinary entry, missing identity and completed identity remain closed.
+2. Navigate all steps, finish and skip, then change tenant/user and deny storage access. =&gt; Ordered targets and labels remain correct; completion is scoped; denied storage permits dismissal and suppresses same-session replay.</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Creation-only eligibility; per-user/tenant isolation; working navigation and dismissal with storage failure.</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>No Agent update
+debug action
+publication or provider request caused by guide.</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Ready creation opens only once; stale/loading/read-only excluded; previous/next bounded; skip and finish recorded; other identities unaffected; storage failure contained; no business callbacks."],"inputs":["entry flag","identity","draft readiness","permission","completion state","denied storage","navigation callbacks"],"unit_boundary":"Real guide component and local preference functions with controlled Tour and editor anchors"}</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":[]}]}</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>vitest</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/agent-creation-guide.test.tsx</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-D1-001</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr"/>
+      <c r="X8" s="5" t="inlineStr"/>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>sha256:9bed58aed86f9578a3896b70744479064c37aeac79986c31c271160363c86fa0</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>sha256:bd0d36fa1d6ac309b24cb9a36355fdae5aaffe2307d5d4d7fd0d8a91e61d3e43</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
           <t>AGENT-LIST-D1-001</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-VIEWS</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-REQ-001
 AGENT-LIST-REQ-002</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-RULE-001
 AGENT-LIST-RULE-002
@@ -895,55 +1998,55 @@
 AGENT-LIST-RULE-005</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Render table view with data-backed agent metadata</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>FE-COMP</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Verify Ant Design table rendering, including header separators and content-based sizing constraints, plus columns, row data, update-time source, and action callbacks without changing the card view contract.</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Render the table with agents containing author, tags, status, and update_time values.
 Render a second agent without update_time but with create_time.</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>{"no_update_agent":{"author":null,"create_time":"2026-09-17T10:30:00","update_time":null},"profile":"mock","updated_agent":{"author":"刘晨","tags":["保健"],"update_time":"2026-09-18T10:30:00"}}</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>1. Render the table with the mocked agent rows. =&gt; The seven columns appear in the specified order in StandardTable backed by Ant Design Table; internal header columns have 1px
 2. Render a row whose update_time is absent and whose create_time is present. =&gt; The update-time cell shows the missing-value placeholder rather than the creation date.
 3. Trigger the row's detail, configure, and publish actions. =&gt; Each callback receives the corresponding agent or numeric agent ID.</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>The table labels include 更新时间 and do not label agents as knowledge bases.
 The table is rendered through StandardTable with the documented typography, backgrounds, 40px rows,
@@ -953,261 +2056,261 @@
 The card component and its data behavior remain unchanged.</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>Do not modify page title, guide area, tabs, or card-mode content.
 Do not add or change backend requests or response contracts.
 Do not fabricate creator or update-time values.</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Table headers render in the required order.","Update time never falls back to create_time.","Missing creator and timestamp values render placeholders.","Action callbacks receive the correct row data.","Header separators are 14px high, vertically centered, and","The scroll wrapper is content-sized with a 500px maximum rather than flex-growing to fill unused space."],"inputs":["agent rows","locale strings","row-action callbacks"],"unit_boundary":"AgentListTable React component with mocked callbacks and translation."}</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr">
+      <c r="S9" s="5" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="T2" s="5" t="inlineStr">
+      <c r="T9" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/run_agent_list_table_test.mjs</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr">
+      <c r="U9" s="5" t="inlineStr">
         <is>
           <t>agentListTable.test.tsx</t>
         </is>
       </c>
-      <c r="V2" s="5" t="inlineStr">
+      <c r="V9" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr"/>
-      <c r="X2" s="5" t="inlineStr"/>
-      <c r="Y2" s="5" t="inlineStr">
+      <c r="W9" s="5" t="inlineStr"/>
+      <c r="X9" s="5" t="inlineStr"/>
+      <c r="Y9" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z2" s="5" t="inlineStr">
+      <c r="Z9" s="5" t="inlineStr">
         <is>
           <t>sha256:42084a90cedb1ae8ffba7cbe7cf1411f12a57a0d42205e6580e12ad08042aeb9</t>
         </is>
       </c>
-      <c r="AA2" s="5" t="inlineStr">
+      <c r="AA9" s="5" t="inlineStr">
         <is>
           <t>sha256:6dd34b7871a706a8b5fc3aa75f7a0dce8d785c1dbc328369e21a9b47cebef59e</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-001</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-013
 CMSR-RULE-014</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Observer emits safe content before stream completion</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Verify bounded marker lookahead and attempt state reset.</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Create an isolated observer and a controlled chunk sequence.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequence":"failed partial, rollback, successful split code and think markers"}</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>1. Feed a safe prefix and pause the source. =&gt; The prefix is emitted before flush or commit.
 2. Roll back the first attempt and feed split markers in the second. =&gt; The second output is ordered and contains no first-attempt residue.</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>The earliest safe content is observable before completion.
 Split markers retain their original semantics.</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O10" s="5" t="inlineStr">
         <is>
           <t>No stale fragment crosses attempts.
 No code is executed by the observer.</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Safe prefix emitted before flush.","Raw code tag retained.","No failed-attempt residue."],"inputs":["normal content","split &lt;think&gt; and &lt;/think&gt;","raw &lt;code&gt; content"],"unit_boundary":"Observer.add_model_new_token and attempt lifecycle"}</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="S10" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="T10" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_model_attempt_stream.py</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr">
+      <c r="U10" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_001</t>
         </is>
       </c>
-      <c r="V3" s="5" t="inlineStr">
+      <c r="V10" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr"/>
-      <c r="X3" s="5" t="inlineStr"/>
-      <c r="Y3" s="5" t="inlineStr">
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr"/>
+      <c r="Y10" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z3" s="5" t="inlineStr">
+      <c r="Z10" s="5" t="inlineStr">
         <is>
           <t>sha256:625e8c8829b51b9cd91344555d05c5ebfdc7bd766d8485eab99b9f22773f3233</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="inlineStr">
+      <c r="AA10" s="5" t="inlineStr">
         <is>
           <t>sha256:242f1aaf8a5fe4427f503e5acb8db2cc6cb5096782c2e4fdf49fcb17ec471420</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-002</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-014
 CMSR-RULE-015</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Running step labels precede reasoning and survive retry rollback</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>FE-COMP</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Verify immediate running labels, rollback preservation, legacy history and removal of terminal label-only cards.</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Create the streaming adapter with a controlled SSE fixture.</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequences":["step 1, failed attempt, rollback, successful raw code, parse","legacy content before step label"]}</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>1. Emit a step label before any model content. =&gt; A running reasoning card displays Step 1 immediately.
 2. Roll back a partial attempt and stream successful raw code. =&gt; Step 1 remains during rollback and only successful raw code follows it.
 3. Parse and reload both new and legacy-order history. =&gt; One code card and one labeled nonempty reasoning card remain; a terminal label-only card is absent.</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>Step label appears before first token.
 Rollback preserves the label.
@@ -1215,326 +2318,326 @@
 Old history prepends late labels.</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>No failed-attempt content.
 No duplicate code card.
 No sibling invocation mutation.</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Running label is visible before content.","Terminal label-only step is hidden.","Successful code is visible after the label before commit.","History equals live output."],"inputs":["step_count","model_attempt_control","model_output_thinking","parse"],"unit_boundary":"Frontend live and history reasoning projection"}</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="S11" s="5" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T11" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_reasoning_card.ts</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U11" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-002</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr"/>
-      <c r="X4" s="5" t="inlineStr"/>
-      <c r="Y4" s="5" t="inlineStr">
+      <c r="W11" s="5" t="inlineStr"/>
+      <c r="X11" s="5" t="inlineStr"/>
+      <c r="Y11" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z4" s="5" t="inlineStr">
+      <c r="Z11" s="5" t="inlineStr">
         <is>
           <t>sha256:b614502639e969ab0f3840d1381f1b12b01cb5b693a0b02d17387192b230b354</t>
         </is>
       </c>
-      <c r="AA4" s="5" t="inlineStr">
+      <c r="AA11" s="5" t="inlineStr">
         <is>
           <t>sha256:03f5fae5200c76ca296c75ab0ebf225f190fb3fe6a7f52c7c8c7e0da2a97d07c</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-003</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-014
 CMSR-RULE-016</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>CoreAgent commits streamed valid semantic repair</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>A protocol-invalid first attempt rolls back while its single preceding step label survives and the corrected result streams and commits.</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>A controlled model yields an invalid response then a pausable valid code action at step one.</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequence":"invalid code, rollback, corrected code chunks, commit, parse"}</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>1. Begin step one and return protocol-invalid model content. =&gt; Exactly one step label precedes begin; the attempt rolls back and one repair is scheduled.
 2. Pause the valid repair after its first safe chunk. =&gt; That chunk is visible before model completion.
 3. Complete the repair and classify it. =&gt; Its attempt commits and a single parse follows.</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>Corrected content is streamed and committed.
 Only the corrected action is executed.
 Lifecycle logs identify the repair without content.</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>No failed content after rollback.
 No repair instruction in user output.
 No suppressed successful stream.</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="P12" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Step label occurs before both model attempts and only once.","Successful repair does not set stream suppression.","Corrected attempt commits once.","Invalid attempt rolls back once."],"inputs":["step one","invalid model content","valid streamed &lt;code&gt; action"],"unit_boundary":"CoreAgent semantic repair and deferred model attempt lifecycle"}</t>
         </is>
       </c>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="R12" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S5" s="5" t="inlineStr">
+      <c r="S12" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T5" s="5" t="inlineStr">
+      <c r="T12" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_semantic_repair_stream.py</t>
         </is>
       </c>
-      <c r="U5" s="5" t="inlineStr">
+      <c r="U12" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_003</t>
         </is>
       </c>
-      <c r="V5" s="5" t="inlineStr">
+      <c r="V12" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr"/>
-      <c r="X5" s="5" t="inlineStr"/>
-      <c r="Y5" s="5" t="inlineStr">
+      <c r="W12" s="5" t="inlineStr"/>
+      <c r="X12" s="5" t="inlineStr"/>
+      <c r="Y12" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z5" s="5" t="inlineStr">
+      <c r="Z12" s="5" t="inlineStr">
         <is>
           <t>sha256:7ef8664f2224d068d7deafecf80f09353d734bc10b35a1147b3cc58d1ae6eacd</t>
         </is>
       </c>
-      <c r="AA5" s="5" t="inlineStr">
+      <c r="AA12" s="5" t="inlineStr">
         <is>
           <t>sha256:1dee7e7ce90f70c40d02907f11be7b55665495fdcaa3dfdec3ab478953c5c38c</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>CMSR-D1-004</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-018</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Rejected model output diagnostics distinguish budget exhaustion without default content leakage</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>SDK-UT</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Correlate each protocol rejection to the model response shape and budget while gating bounded raw previews.</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Use isolated model diagnostics for a reasoning-only length response and a malformed nonempty response.</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","responses":["length with 4096 reasoning-only output tokens","malformed nonempty code Action"]}</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>1. Reject a reasoning-only length response with diagnostics disabled. =&gt; The log records model, attempt, requested and consumed tokens, reasoning and content counts, and reasoning-only budget exhaustion without raw text.
 2. Reject a malformed content response. =&gt; The distinct protocol reason and response shape are logged under its own attempt identifier.
 3. Enable diagnostic content preview for a rejected response longer than the preview cap. =&gt; Only a single escaped bounded prefix of model content and reasoning is logged; the full text remains absent.</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>Each rejection is attributable to one attempt and specific failure class.
 Raw output is absent by default and bounded on explicit opt-in.</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr">
         <is>
           <t>No model output or user prompt enters SSE or persisted history from diagnostics.
 No secret or full raw payload is logged by default.
 No retry-budget or execution behavior changes.</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>{"assertions":["Reasoning-only budget exhaustion flag is accurate.","Logs include attempt and token counts.","Default logs omit raw content.","Opt-in previews are escaped and capped."],"inputs":["finish_reason=length","reasoning_content","invalid code Action","explicit diagnostic flag"],"unit_boundary":"OpenAI model response diagnostics and CoreAgent protocol-error logging"}</t>
         </is>
       </c>
-      <c r="Q6" s="5" t="inlineStr"/>
-      <c r="R6" s="5" t="inlineStr">
+      <c r="Q13" s="5" t="inlineStr"/>
+      <c r="R13" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S6" s="5" t="inlineStr">
+      <c r="S13" s="5" t="inlineStr">
         <is>
           <t>pytest</t>
         </is>
       </c>
-      <c r="T6" s="5" t="inlineStr">
+      <c r="T13" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_protocol_rejection_diagnostics.py</t>
         </is>
       </c>
-      <c r="U6" s="5" t="inlineStr">
+      <c r="U13" s="5" t="inlineStr">
         <is>
           <t>test_cmsr_d1_004</t>
         </is>
       </c>
-      <c r="V6" s="5" t="inlineStr">
+      <c r="V13" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W6" s="5" t="inlineStr"/>
-      <c r="X6" s="5" t="inlineStr"/>
-      <c r="Y6" s="5" t="inlineStr">
+      <c r="W13" s="5" t="inlineStr"/>
+      <c r="X13" s="5" t="inlineStr"/>
+      <c r="Y13" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z6" s="5" t="inlineStr">
+      <c r="Z13" s="5" t="inlineStr">
         <is>
           <t>sha256:9f06a6565fff8e542fdcb89725b5fc7f669ad52b07301bdc99aa3e2eba23552c</t>
         </is>
       </c>
-      <c r="AA6" s="5" t="inlineStr">
+      <c r="AA13" s="5" t="inlineStr">
         <is>
           <t>sha256:a53056127d5f2efce4a9d98c92c9c97892451de0d1d353603584612c0a9ef1ba</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA6"/>
+  <autoFilter ref="A1:AA13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2175,12 +3278,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -2347,21 +3450,460 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>AGENT-CONFIG-D4-001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-REQ-002
+AGENT-CONFIG-REQ-003</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-RULE-001
+AGENT-CONFIG-RULE-002
+AGENT-CONFIG-RULE-003
+AGENT-CONFIG-RULE-004
+AGENT-CONFIG-RULE-005
+AGENT-CONFIG-RULE-006
+AGENT-CONFIG-RULE-007
+AGENT-CONFIG-RULE-008
+AGENT-CONFIG-RULE-009
+AGENT-CONFIG-RULE-010
+AGENT-CONFIG-RULE-011</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Configure an empty draft through the measured editor without losing save or permission gates</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Prove actual desktop geometry, internal scrolling, actionable resources, question boundary, autosaved edits and validation/read-only outcomes in one deterministic browser journey.</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>A local frontend is running and all backend/provider HTTP requests are routed to deterministic logical fixtures.
+Logical fixtures expose an editable draft, an empty draft, resource/model choices, and a read-only draft; updates are captured only in fixture state.
+A populated fixture exposes selected tools plus a managed knowledge tool and selected internal/external child Agents with real catalog labels and saved version snapshots; knowledge-base rows use the current fixture presentation.</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>{"constrained_viewport":{"height":800,"width":1280},"editable_draft":{"asset_ref":"empty_agent_draft"},"geometry_tolerance_px":1,"profile":"mock","read_only_draft":{"asset_ref":"read_only_agent_draft"},"selected_child_agents":{"asset_ref":"selected_internal_external_agents_with_saved_versions"},"selected_row":{"action_glyph_size":14,"action_target_size":24,"border_color":"#DFDFDF","child_avatar_size":32,"gap":8,"height":48,"horizontal_padding":12,"name_color":"#191919","name_font_size":14,"name_font_weight":400,"name_line_height":22,"radius":4,"tag_color":"#777777","tag_font_size":12,"tag_line_height":18,"tool_icon_size":24,"vertical_padding":8},"selected_tools":{"asset_ref":"selected_tools_with_managed_knowledge_tool"},"viewport":{"height":1080,"width":1920}}</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the initialized editable empty draft at the desktop reference viewport. =&gt; Navigation64px, conversation561px, remaining configuration1295px fit the1920px viewport without horizontal overflow; tab64px and identity74px precede four white radius8 cards with gap12 and no universal outer stroke/shadow.
+2. Inspect the empty card/resource geometry and selected title/description styles. =&gt; Basic/model empty reference heights are224/268px where reference children apply; avatar preview is100px, basic columns share width equally with16px gap and description textarea is100px; resources share one card in knowledge/welcome/skills/tools/child order, add row is two columns gap8 with a left48px entry and3% dark background, titles16px/24px weight500
+3. Scroll to lower resources/advanced controls, collapse and reopen a resource, and open add-resource selection separately from create/manage. =&gt; Scrolling stays inside the configuration pane and identity/action controls remain reachable; no association update occurs before selection confirmation, and model/prompt/guardrail capabilities remain reachable.
+4. Edit a greeting and add/edit five preset questions, then attempt another addition and remove one. =&gt; Existing update payloads retain edited values; addition disables at five and re-enables below five without writes from initial render.
+5. Invoke debug/publication with missing required data, then provide valid required fields and wait for autosave before invoking debug/publication entry again. =&gt; Validation prevents downstream actions for invalid data; valid debug/publication entry follows existing validation/idle-save flow and publication modal, without publishing to a real backend.
+6. Reopen captured fixture draft, then load a read-only fixture and resize to the constrained viewport. =&gt; Saved edits remain visible, read-only prevents edits/publication, controls stay usable without horizontal overflow or clipped populated content.
+7. Open model, knowledge, skill, tool and child-Agent association entries, inspect the right drawer and close each without edits. =&gt; All five entries reuse the shared right drawer; association data and existing save count remain unchanged.
+8. Open the populated fixture and inspect selected tools, child Agents, add-entry order and the existing knowledge-base row at desktop and constrained widths, then resize below the small-screen breakpoint. =&gt; Tools/child Agents use two equal columns with8px gaps and48px white rows with4px radius,1px#DFDFDF border,12px/8px padding and the current knowledge shell shadow; names are14px/22px regular400#191919 with ellipsis/full-name tooltips, real neutral tags are12px/18px#777777 and8px from the name, marks/avatars are24px/32px, and14px action glyphs stay visible in24px targets. The add entry follows all selected rows; below sm the grid uses one column without horizontal overflow. Knowledge rows and selector drawers retain their existing presentation.
+9. Open a selected tool configuration, inspect a saved child-version tooltip, remove one selected tool and one internal child Agent, wait for fixture autosave, then reopen the captured draft and repeat mutation attempts with a read-only populated fixture. =&gt; Existing configuration prerequisites and saved version metadata remain reachable; only the intended tool/child selection is removed and persisted through existing fixture payloads, the managed knowledge tool and other child snapshots remain intact, and read-only controls prevent mutation. Initial rendering and tooltip inspection generate no association writes.</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>Desktop measured layout fits the available box model with at most1px geometry tolerance rather than hardcoding overflowing source widths.
+Four cards/resources use the measured geometry and numeric typography; unavailable font glyph parity is not claimed.
+Question addition uses maximum five and edited data persists only through existing fixture update contracts.
+Validation/save/permission gates and model/resource/guardrail reachability survive regrouping.
+Lower content scrolls internally and workflow actions remain reachable across viewport sizes.
+All five association drawers open and close without association writes; existing configuration/selection controllers remain reachable.
+Populated tools/child Agents match the frozen selected-row numerical contract, resource/add ordering and responsive layout while current knowledge rows/drawers retain their presentation.
+Existing selected-resource configuration/removal and saved-version tooltips work; captured/reopened fixture state retains managed knowledge tools and unaffected selections, and read-only disables mutations.</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Do not call a real backend/provider, publish a real version, create real resources, or introduce a new endpoint.
+Do not write from render/collapse, silently truncate legacy data, or bypass read-only/validation/save gates.
+Do not fabricate optional metadata, discard managed knowledge tools or retained child versions, or change current knowledge/drawer presentation.</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>{"actor":"Agent editor user","failure_evidence":["Failure screenshot/trace plus violated geometry or control assertion.","Sanitized captured update payloads and unexpected request paths.","Missing controls, clipped content, or mismatched saved fixture values."],"final_business_result":["The user can configure an empty draft in the measured layout while keeping saved edits and existing workflow gates.","All mutations remain inside deterministic fixture state.","Populated selected tools and child Agents use consistent compact rows and retain their configuration/removal permissions and saved association data."],"journey":["Open an existing empty draft and inspect desktop composition.","Associate resources through the existing selection path and edit conversation guidance.","Wait for fixture autosave and invoke permission/validation guarded workflows.","Reopen fixture data and inspect a read-only/narrow-screen state.","Inspect populated tool/child rows, configure/remove selected resources, and reopen the saved fixture state while preserving knowledge associations and child versions."]}</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["http-fixture"]}],"timeout_seconds":120}</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d4/agent-config-layout.spec.mjs</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CONFIG-D4-001</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>http-fixture</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr"/>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>sha256:5838edebe9452e43ecb1c573cd00bd5a64fd2f0562891f93f5bc4cefefc2258d</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>sha256:67c8065cd1d5e5b2799cfb3688fd415858844226268e2704b60abb314c143d2e</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-D4-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-LAYOUT</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-REQ-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-RULE-001
+AGENT-DEBUG-RULE-002
+AGENT-DEBUG-RULE-003</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Debug a draft in measured layout through preserved runtime and panel controls</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Prove browser geometry and a complete deterministic question/send/stop/clear/layout journey without real writes or providers.</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Local frontend running; all API requests intercepted by deterministic draft/model/chat fixtures.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"constrained_viewport":{"height":800,"width":1280},"draft":{"asset_ref":"debug_agent_draft"},"geometry_tolerance_px":1,"profile":"mock","viewport":{"height":1080,"width":1920}}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Open a valid draft and invoke its guarded debug workflow. =&gt; Common tabs and identity remain above both panes; debug width488, padding24, gap10 and card-aligned top with measured header/welcome/question/composer styles.
+2. Select a question and send it through the mocked debug stream, then stop an active run. =&gt; Selection fills exact composer text without a request; send uses existing debug run payload and stop is reachable through existing cancel behavior.
+3. Maximize and restore, clear conversation, toggle comparison and close/reopen debug. =&gt; Layout changes retain existing conversation; clear restores welcome; comparison stays reachable; reopen retains mounted local state.
+4. Resize to constrained viewport and inspect default-chat presentation separately with deterministic fixtures. =&gt; No horizontal page overflow, internal welcome/messages scrolling and controls reachable; default chat has no debug geometry or disclaimer.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Measured desktop geometry within1px; deterministic chat and local controls work; responsive layout retains controls; default presentation unaffected.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No real provider/backend call; no configuration writes from selection or panel controls; no new endpoint; no bypass of existing guarded debug entry.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"actor":"Agent editor user","failure_evidence":["Failure screenshot and trace","violated geometry or runtime assertion","unexpected HTTP writes"],"final_business_result":["User can debug the current draft in measured presentation while preserving runtime and configuration state."],"journey":["Open draft","invoke debug","select and send question","stop run","change pane layout","clear","compare and resize"]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["http-fixture"]}],"timeout_seconds":120}</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d4/agent-debug-layout.spec.mjs</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-DEBUG-D4-001</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>http-fixture</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:de5e7b33a4bed63c56e6b36a2549125842c1b44e30dbf0ccca5d7945479067d2</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:af5ff413a111fd51e3603dc72918f0677aec883a21cb38802a9aba321197dd6e</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-D4-001</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-CREATION-GUIDE</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-REQ-001</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-RULE-001
+AGENT-GUIDE-RULE-002
+AGENT-GUIDE-RULE-003</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Create an Agent and complete or skip its measured first-creation guide</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Prove complete creation-to-editor tour journey, geometry, remembered dismissal and safe responsive/read-only behavior.</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Local frontend running; HTTP intercepted by deterministic authenticated editable draft and creation fixtures; isolated preference storage.</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>{"constrained_viewport":{"height":800,"width":1280},"draft":{"asset_ref":"newly_created_agent"},"geometry_tolerance_px":1,"profile":"mock","viewport":{"height":1080,"width":1920}}</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>1. Open Agent list, create a named draft and enter editor. =&gt; One mocked creation succeeds; first guide appears only after correct draft load; measured body/type/padding/buttons/shadow and assistant highlight.
+2. Navigate next and previous through core, resources and workflow steps, then choose Start creation. =&gt; Exact four titles/descriptions and matching highlights/arrows; measured popovers within1px; final dismisses and focuses composer without draft updates or run/publication.
+3. Reload completed route, open ordinary editor, then reset local preference and skip a fresh creation entry. =&gt; Completed and ordinary routes do not replay; skip suppresses replay after reload.
+4. Open read-only marked route and a fresh editable route at constrained viewport. =&gt; Read-only has no guide; constrained steps keep buttons in viewport with no horizontal page overflow.</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>Full creation and four-step journey; source geometry within1px; remembered skip/finish; read-only exclusion and reachable constrained layout.</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>No real backend/provider invocation; no Agent update after initial mocked create; no debug or publish call caused by tour.</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>{"actor":"First-time Agent creator","failure_evidence":["Failure screenshot/trace","incorrect title or target","violated geometry","unexpected HTTP writes"],"final_business_result":["User understands configuration workflow and can start editing the created draft after completion or dismissal."],"journey":["Open Agent list","create draft","advance and return through guide","finish","reload","skip","check read-only and constrained viewport"]}</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["http-fixture"]}],"timeout_seconds":120}</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d4/agent-creation-guide.spec.mjs</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-GUIDE-D4-001</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>http-fixture</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr"/>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>sha256:b90762e85a71ff0d88345201247c01a559a1aff624324338c8b80a9604de96eb</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>sha256:270648d673d9a74ec8aaa588c8415414cc5e8020ba7b84d7b04567344d43b723</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
           <t>AGENT-LIST-D4-001</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-VIEWS</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-REQ-001
 AGENT-LIST-REQ-002</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>AGENT-LIST-RULE-001
 AGENT-LIST-RULE-002
@@ -2370,47 +3912,47 @@
 AGENT-LIST-RULE-005</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Switch between the agent card and table presentations</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>E2E</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Verify Ant Design table separators and content-responsive sizing at desktop and constrained viewport widths, and confirm that table view retains existing list workflows.</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Open the agent list with at least two mocked agents, including one with update_time and one without it.</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>{"agent_count":8,"profile":"mock","viewport":{"height":1080,"width":1920}}</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>1. Switch from card mode to table mode. =&gt; The page heading, guide, and tabs remain unchanged while the table and its pagination appear.
 2. Verify columns and representative row values. =&gt; The column order is 名称、类型、描述、状态、创建人、更新时间、操作; timestamps reflect update_time only.
@@ -2418,7 +3960,7 @@
 4. Search for an agent, activate its configure action, then return and switch back to card mode. =&gt; Search and navigation still work, and the card presentation returns with its prior layout and metadata.</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>At 1920×1080 the table occupies the measured 1807px content width; its height follows its rendered rows, grows no higher than 500px, and does not fill unused space.
 The table uses StandardTable with 14px/#191919/0px typography, white rows, a
@@ -2428,79 +3970,79 @@
 Page-level content above the list and existing card mode are unchanged.</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>No backend API or data mutation is introduced by switching views.
 Do not use create_time as update_time.
 Do not add body vertical separators or an outer table border; header separators remain centered and shorter than the 40px header cell.</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>{"actor":"Agent list user","failure_evidence":["Missing/incorrect table headings or row values.","Search, navigation, pagination, or view switching fails.","The table changes content above the list or mutates agent data."],"final_business_result":["The same agent collection remains available in either presentation.","Existing list operations remain reachable."],"journey":["Open the agent list.","Switch between card and table modes.","Search and open an agent configuration."]}</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>implemented</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>custom</t>
         </is>
       </c>
-      <c r="T2" s="5" t="inlineStr">
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>test/automation/d4/run_agent_list_views_e2e.mjs</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr">
+      <c r="U5" s="5" t="inlineStr">
         <is>
           <t>agent-list-high-fidelity.spec.ts</t>
         </is>
       </c>
-      <c r="V2" s="5" t="inlineStr">
+      <c r="V5" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr"/>
-      <c r="X2" s="5" t="inlineStr"/>
-      <c r="Y2" s="5" t="inlineStr">
+      <c r="W5" s="5" t="inlineStr"/>
+      <c r="X5" s="5" t="inlineStr"/>
+      <c r="Y5" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z2" s="5" t="inlineStr">
+      <c r="Z5" s="5" t="inlineStr">
         <is>
           <t>sha256:1093e9eea123f868058b2922bcb8becb7058e0378301e97276df51156c4ba9fc</t>
         </is>
       </c>
-      <c r="AA2" s="5" t="inlineStr">
+      <c r="AA5" s="5" t="inlineStr">
         <is>
           <t>sha256:a905ec4d8fcce1e93354988f937f8f560872b64738f762662e6250e2413b9b8b</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CMSR-D4-001</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>CMSR-005</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>CMSR-RULE-013
 CMSR-RULE-014
@@ -2508,48 +4050,48 @@
 CMSR-RULE-016</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Browser shows retry output incrementally without blank steps</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>E2E</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>automated</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Verify a user sees only successful raw code and one executed action in a real conversation.</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>A local Nexent instance
 test tenant and controllable model provider are configured.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>{"profile":"mock","sequences":["failed transport partial then success","step-one invalid protocol then valid paused repair"]}</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>1. Open Agent chat and send the fixed prompt. =&gt; Step 1 appears before the first model token; the first partial output is then rolled back while the label remains.
 2. Pause the second provider response after its first safe fragment. =&gt; The reasoning card displays the successful raw fragment before provider completion.
@@ -2557,7 +4099,7 @@
 4. Repeat in a new conversation with semantic repair at step one. =&gt; Corrected raw code is visible during the pause and after refresh; Connecting does not persist.</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Running Step 1 is visible before content.
 No terminal label-only reasoning card.
@@ -2565,59 +4107,59 @@
 Refreshed history matches the final UI.</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>No failed partial text after rollback.
 No duplicate execution card.</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>{"actor":"Authenticated test tenant user","failure_evidence":["Retain browser screenshot","network timing and console trace on failure."],"final_business_result":["Only the committed attempt and its single executed code action are visible."],"journey":["Open the Agent conversation.","Trigger controlled retry.","Observe streaming.","Reload and inspect history."]}</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>{"profiles":[{"name":"mock","required_services":["model-provider"]}]}</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="R6" s="5" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr"/>
-      <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="5" t="inlineStr"/>
-      <c r="V3" s="5" t="inlineStr">
+      <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr"/>
+      <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6" s="5" t="inlineStr">
         <is>
           <t>mock</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr">
+      <c r="W6" s="5" t="inlineStr">
         <is>
           <t>model-provider</t>
         </is>
       </c>
-      <c r="X3" s="5" t="inlineStr"/>
-      <c r="Y3" s="5" t="inlineStr">
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
         <is>
           <t>校验通过</t>
         </is>
       </c>
-      <c r="Z3" s="5" t="inlineStr">
+      <c r="Z6" s="5" t="inlineStr">
         <is>
           <t>sha256:f110f582fe091286fdaa5301f8bdc22703bf583fc7c6c95214ae8c8187a612a1</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="inlineStr">
+      <c r="AA6" s="5" t="inlineStr">
         <is>
           <t>sha256:4f53cda18c2baa0c0354bb5f9a3ecbe5ed12ab4d8e11ba873c2f11161202b945</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA3"/>
+  <autoFilter ref="A1:AA6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(agent): commit accepted streamed code action repairs
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -1143,12 +1143,13 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>A controlled model yields an invalid response then a pausable valid code action at step one.</t>
+          <t>Protocol repair retry is enabled for the controlled Agent.
+A controlled model yields an invalid response then a pausable repair at step one.</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>{"profile":"mock","sequence":"invalid code, rollback, corrected code chunks, commit, parse"}</t>
+          <t>{"profile":"mock","sequence":"invalid code, rollback, pausable corrected code or clarification, commit; invalid code or clarification rolls back","suppression_capabilities":[true,false]}</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
@@ -1174,7 +1175,7 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Step label occurs before both model attempts and only once.","Successful repair does not set stream suppression.","Corrected attempt commits once.","Invalid attempt rolls back once."],"inputs":["step one","invalid model content","valid streamed &lt;code&gt; action"],"unit_boundary":"CoreAgent semantic repair and deferred model attempt lifecycle"}</t>
+          <t>{"assertions":["Step label occurs before both model attempts and only once.","Successful repair does not set stream suppression.","Corrected attempt commits once.","Invalid attempt rolls back once.","Invalid repair rolls back without execution.","Accepted clarification commits before interaction."],"inputs":["step one","invalid model content","valid streamed &lt;code&gt; action"],"unit_boundary":"CoreAgent semantic repair and deferred model attempt lifecycle"}</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr"/>
@@ -1212,12 +1213,12 @@
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
-          <t>sha256:7ef8664f2224d068d7deafecf80f09353d734bc10b35a1147b3cc58d1ae6eacd</t>
+          <t>sha256:c3d470f2b34d64b77b32c4e7f56e0ba90a1342dfe28fdbdfbdd1879bc008119d</t>
         </is>
       </c>
       <c r="AA4" s="5" t="inlineStr">
         <is>
-          <t>sha256:1dee7e7ce90f70c40d02907f11be7b55665495fdcaa3dfdec3ab478953c5c38c</t>
+          <t>sha256:cb7b08a8985cb407cb19b796efbc05df45c6cedd57b1deca1fe187ad199c9e51</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1664,7 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:570d7db5b7480c6b3a3a3adcc953158f7c496e44a79e90ad1ca3a4df676d573f</t>
+          <t>sha256:f8f1bc3e7a01d6ffd739d9fbe695e28533e4c410847a09b6405a7dbd4c2e948a</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: defer Docker startup for official tool actions
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_D5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_D2'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_D5'!$A$1:$AA$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_D5'!$A$1:$AA$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
@@ -551,11 +551,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -646,8 +646,52 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Official tool fast path with deferred Docker initialization</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>All Docker-configured Agents can execute approved simple tool steps locally before creating their ordinary executor.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-001
+TFP-RULE-002
+TFP-RULE-003
+TFP-RULE-004
+TFP-RULE-005</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>D1
+D3
+D4
+D5</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>{"requirement_ids":["TFP-001"],"spec_path":"nexent-doc/docs/Developing/runtime-sandbox-tool-fastpath/proposal.md"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -658,13 +702,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -679,9 +723,9 @@
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="29" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -1351,8 +1395,810 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D1-001</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-001
+TFP-RULE-005</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Simple official tool steps and final answers never acquire Docker</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Simple official tool steps and final answers never acquire Docker</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>1. Execute assignment, print and final_answer using an approved official tool. =&gt; The value, logs and final flag match the local interpreter.
+2. Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Factory acquisition and warm-up counts are zero.
+The wrapped tool is called once and final_answer returns the saved result.
+Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request.</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>No Docker bridge, container or kernel is created.</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Factory acquisition and warm-up counts are zero.","The wrapped tool is called once and final_answer returns the saved result.","Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request."],"inputs":["Simple official tool steps and final answers never acquire Docker"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>pytest
+pytest</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath_aidp.py</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d1_001
+test_tfp_d1_001_aidp</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:f49d99ec8a0bad9223bdd15df090912a0a2c67816b5857d6add0a9fbd42f851c</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:01d39055c92bd0c0fe6e4360ed1345a6eae93173d20da7f1fea830c15a61839e</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D1-002</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-002</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Full-step admission prevents partial local execution</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Full-step admission prevents partial local execution</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>1. Submit a tool call followed by an import, an unapproved call or a bare data expression outside assignment and call arguments. =&gt; The whole step is delegated before any local call.
+2. An aidp_search step followed by ordinary code makes no provider request before whole-step delegation. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Mixed code is passed once to the original executor.
+No approved tool is called by the fast path before delegation.
+An aidp_search step followed by ordinary code makes no provider request before whole-step delegation.</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>No partial execution or tool replay.</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Mixed code is passed once to the original executor.","No approved tool is called by the fast path before delegation.","An aidp_search step followed by ordinary code makes no provider request before whole-step delegation."],"inputs":["Full-step admission prevents partial local execution"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>pytest
+pytest</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath_aidp.py</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d1_002
+test_tfp_d1_002_aidp</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" s="5" t="inlineStr"/>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:45bd2b9559253a21e4b96e995b91daa065ff8f9ea28bf3c3908b9756b5791782</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:01d39055c92bd0c0fe6e4360ed1345a6eae93173d20da7f1fea830c15a61839e</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D1-003</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-003</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Promotion preserves user values and remains sticky</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Promotion preserves user values and remains sticky</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>1. Produce aliased user containers and a tool result, then submit ordinary code. =&gt; One executor is initialized and receives the user namespace.
+2. Submit another approved step. =&gt; The initialized executor is reused.</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Values and shared container references survive migration.
+Internal interpreter state and tool objects are not migrated.
+The factory is called once.</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>No repeated prior tool invocation.</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Values and shared container references survive migration.","Internal interpreter state and tool objects are not migrated.","The factory is called once."],"inputs":["Promotion preserves user values and remains sticky"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_tool_fastpath.py</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d1_003</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr"/>
+      <c r="X8" s="5" t="inlineStr"/>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>sha256:78c3f112432755e552f23bdb788339f518f550d911228d013071fc2c932db42d</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>sha256:fba0f34909d32b214bd0a02edc0f4c28eaf34e88e682b3977a2f5a6ea22a64cb</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D1-004</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-002</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Tool identity cannot be forged by names or sources</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Tool identity cannot be forged by names or sources</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>1. Provide an exact official tool, an unknown subclass, a same-name custom tool and an MCP source. =&gt; Only the approved official source and exact implementation qualify.
+2. Only exact AidpSearchTool from the local source qualifies; MCP, custom, subclass and IndependentAidpSearchTool identities cannot impersonate aidp_search. Explicit omission from the allowlist delegates. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Unapproved identities delegate to the original executor.
+Reserved names and callable aliases do not qualify.
+Only exact AidpSearchTool from the local source qualifies; MCP, custom, subclass and IndependentAidpSearchTool identities cannot impersonate aidp_search. Explicit omission from the allowlist delegates.</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>No unauthorized local invocation.</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Unapproved identities delegate to the original executor.","Reserved names and callable aliases do not qualify.","Only exact AidpSearchTool from the local source qualifies; MCP, custom, subclass and IndependentAidpSearchTool identities cannot impersonate aidp_search. Explicit omission from the allowlist delegates."],"inputs":["Tool identity cannot be forged by names or sources"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>pytest
+pytest</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath_aidp.py</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d1_004
+test_tfp_d1_004_aidp</t>
+        </is>
+      </c>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr"/>
+      <c r="X9" s="5" t="inlineStr"/>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z9" s="5" t="inlineStr">
+        <is>
+          <t>sha256:2c10e437ccb446a0554d12e76188babbe4d97d0bffc4fd19f98498a86a05c17a</t>
+        </is>
+      </c>
+      <c r="AA9" s="5" t="inlineStr">
+        <is>
+          <t>sha256:01d39055c92bd0c0fe6e4360ed1345a6eae93173d20da7f1fea830c15a61839e</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D1-005</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-004</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Exceptions, cancellation and cleanup are safe</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Exceptions, cancellation and cleanup are safe</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>1. Fail an approved tool, close an unused wrapper, fail workspace or variable initialization and cancel during acquisition. =&gt; No failed call is replayed and acquired resources close once.
+2. AIDP provider errors propagate without acquiring or replaying through Docker. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Local errors do not trigger remote replay.
+Cleanup is idempotent.
+Cancellation before execution prevents tool calls and releases acquired resources.
+AIDP provider errors propagate without acquiring or replaying through Docker.</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>No initialization during cleanup.
+No execution after cancellation.</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Local errors do not trigger remote replay.","Cleanup is idempotent.","Cancellation before execution prevents tool calls and releases acquired resources.","AIDP provider errors propagate without acquiring or replaying through Docker."],"inputs":["Exceptions, cancellation and cleanup are safe"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>pytest
+pytest
+pytest</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath_aidp.py</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d1_005
+test_tfp_d1_005_deferred_setup
+test_tfp_d1_005_aidp</t>
+        </is>
+      </c>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr"/>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>sha256:f9b9a844e326fc8cac16cb7fa2c69d2ea2f5604696c678c814dfa2ff0058d915</t>
+        </is>
+      </c>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>sha256:e263aa60250b6329f8943aaa6a2f8f0be1b27c3a8dcdfc7364eff56c8ededcaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D1-006</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-001
+TFP-RULE-004
+TFP-RULE-005</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Factory defers initialization and prepares promoted workspaces</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Factory defers initialization and prepares promoted workspaces</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>1. Construct a root and child with Docker fast paths and omit the SDK enablement argument. =&gt; Both remain uninitialized.
+2. Activate root and child ordinary executors. =&gt; The session group is shared and each workspace is initialized when its executor appears.
+3. Omit the deployment enablement flag and SDK run-info field, then repeat with an explicit false flag. Exercise MCP and non-MCP run construction. =&gt; Omitted flags enable deferred execution; explicit false retains eager initialization in both paths. Default allowlists include AidpSearchTool, and explicit allowlists retain their configured contents.</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Disabled mode keeps eager initialization.
+Omitted deployment and SDK flags enable the deferred Docker path, including missing-field fallbacks in MCP and non-MCP run construction.
+Enabled mode delays warm-up and script binding until activation.
+Workspace synchronization precedes ordinary code.
+Actual executors release exactly once.
+Deployment and SDK default allowlists include AidpSearchTool; explicit allowlists and explicit false opt-out remain respected.</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>No kernel for unused child.
+No duplicated session container.</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Disabled mode keeps eager initialization.","Omitted deployment and SDK flags enable the deferred Docker path, including missing-field fallbacks in MCP and non-MCP run construction.","Enabled mode delays warm-up and script binding until activation.","Workspace synchronization precedes ordinary code.","Actual executors release exactly once.","Deployment and SDK default allowlists include AidpSearchTool; explicit allowlists and explicit false opt-out remain respected."],"inputs":["Factory defers initialization and prepares promoted workspaces"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>pytest
+pytest
+pytest
+pytest</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath_defaults.py</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d1_006
+test_tfp_d1_006_backends
+test_tfp_d1_006_configuration
+test_tfp_d1_006_run_defaults</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W11" s="5" t="inlineStr"/>
+      <c r="X11" s="5" t="inlineStr"/>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z11" s="5" t="inlineStr">
+        <is>
+          <t>sha256:2bd5d2095842fbb8b4a21db9116ddf8f82a85adfd71351b5084d0d8005a387dc</t>
+        </is>
+      </c>
+      <c r="AA11" s="5" t="inlineStr">
+        <is>
+          <t>sha256:071883550d50b75dd6588a75d883d5af51a92b6edadbf1c02b30412179705beb</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA5"/>
+  <autoFilter ref="A1:AA11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1653,7 +2499,7 @@
       <c r="X2" s="5" t="inlineStr"/>
       <c r="Y2" s="5" t="inlineStr">
         <is>
-          <t>校验通过</t>
+          <t>实现哈希失效</t>
         </is>
       </c>
       <c r="Z2" s="5" t="inlineStr">
@@ -1679,7 +2525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1981,8 +2827,136 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D3-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-001
+TFP-RULE-003
+TFP-RULE-005</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Real Nexent runtime defers Docker until ordinary code</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-IT</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Real Nexent runtime defers Docker until ordinary code</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>A disposable Nexent deployment with this implementation and an approved controlled provider profile is available.
+The current sandbox image has its sandbox user and a reachable kernel service.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Run an approved knowledge query with a controlled model. =&gt; No kernel or warm-up appears.
+2. Run retrieval followed by ordinary Python and a script-produced artifact. =&gt; The saved variable is available and the artifact is downloadable.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Correct final answer and persisted tool events.
+One activation per Agent needing ordinary code.
+All run resources are reclaimed.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No duplicate tool call or cross-tenant access.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"cleanup":["Remove disposable conversations and artifacts; release run kernels."],"integration_boundary":["Running Nexent API, SDK model loop, official tools, Docker kernel and artifact storage"],"observations":["Executor acquisition counters, warm-up traces, tool events, variable consumption and downloaded artifact"]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["model-provider"]},{"name":"real_smoke","required_services":["model-provider"]}]}</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock
+real_smoke</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>model-provider</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:d0707e473b4368889ed27687c15f63d454b843ff2296508357797058551c52f3</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:4f53cda18c2baa0c0354bb5f9a3ecbe5ed12ab4d8e11ba873c2f11161202b945</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1993,7 +2967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2294,8 +3268,134 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D4-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-001
+TFP-RULE-003
+TFP-RULE-005</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Chat displays fast and promoted tool tasks correctly</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Chat displays fast and promoted tool tasks correctly</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>A disposable Nexent deployment with this implementation and an approved controlled provider profile is available.
+A disposable authenticated browser session and a working current sandbox image are available.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Open a disposable Agent chat and request a knowledge answer. =&gt; A single tool event and correct final answer appear.
+2. Request a task requiring Python and reload the conversation. =&gt; The task completes and history preserves the result without duplicates.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>The final answer and artifact are accessible.
+Refreshed history matches the live result.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No duplicate tool card or stale sibling output.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"actor":"Authenticated disposable tenant user","failure_evidence":["Retain Playwright trace, screenshot and network evidence on failure."],"final_business_result":["Both task types complete with correct visible output."],"journey":["Open chat.","Run approved tool task.","Run ordinary Python task.","Reload history and download artifact."]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["model-provider"]}]}</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>model-provider</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:82e008044b9a89dd07a01bdb8aba0553d5b2d2b173758d98b3011e370e0f6463</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:4f53cda18c2baa0c0354bb5f9a3ecbe5ed12ab4d8e11ba873c2f11161202b945</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2306,7 +3406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2326,10 +3426,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -2599,8 +3699,262 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D5-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-002</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Untrusted syntax and hostile tool identities cannot enter the local path</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>SECURITY</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Untrusted syntax and hostile tool identities cannot enter the local path</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Submit attributes, imports, alias calls, unpacking, loops and reserved-variable assignments, including initial variables that shadow tool or framework call names. =&gt; All are rejected before execution.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Zero local tool calls for all rejected inputs.
+The full source is delegated unchanged.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No host file, shell or reflection operation is executed.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"condition":["Controlled hostile source and same-name tool fixtures."],"metrics":["Local invocation count.","Admission result."],"recovery_expectations":["A later valid step can still use the ordinary executor."],"risk":"A permissive fast-path validator could allow arbitrary host code.","risk_type":"SECURITY","thresholds":["Zero unauthorized local invocations.","Every hostile sample rejects admission."]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d5/test_tool_fastpath_risks.py</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d5_001</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:cad74b7982db6a898f9267891d908d5e4a026fff456b4e16172e26fa1f499f08</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:6af5717e8cd49952880712aeb98f89e5242c74430374ce491d472e1f80f687cc</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>TFP-D5-002</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>TFP-001</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>TFP-RULE-001
+TFP-RULE-004</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Repeated simple actions avoid startup and cleanup overhead</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Repeated simple actions avoid startup and cleanup overhead</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Use isolated official tool instances and a controlled executor factory.</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>1. Run one thousand small approved steps, then close the wrapper twice. =&gt; No ordinary executor is created and every intended tool call occurs once.</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>Factory count is zero.
+All one thousand results are correct.
+P95 local route time is at most 10 ms for small fixtures.</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>No kernel, bridge or container created by the fast-path wrapper.</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>{"condition":["One thousand warmed steps smaller than 4 KiB with a controlled immediate official tool."],"metrics":["Factory call count.","Per-step P95 duration."],"recovery_expectations":["Cleanup remains idempotent and does not acquire resources."],"risk":"Interpreter routing could erase the saved sandbox startup cost.","risk_type":"PERFORMANCE","thresholds":["Factory count equals zero.","P95 is at most 10 ms excluding provider and tool I/O."]}</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d5/test_tool_fastpath_risks.py</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>test_tfp_d5_002</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" s="5" t="inlineStr"/>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>sha256:29bfd14fe4f25184e0320e677b23279765cab9691cf05c6bbf44e76dc8bd0e73</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>sha256:6af5717e8cd49952880712aeb98f89e5242c74430374ce491d472e1f80f687cc</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test(agent): verify repaired streams in deployed runtime and browser
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -1700,10 +1700,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
     <col width="17" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -1948,12 +1948,24 @@
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="S2" s="5" t="inlineStr"/>
-      <c r="T2" s="5" t="inlineStr"/>
-      <c r="U2" s="5" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d3/test_semantic_repair_runtime.py</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>test_cmsr_d3_001</t>
+        </is>
+      </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
           <t>mock
@@ -1978,7 +1990,7 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:4f53cda18c2baa0c0354bb5f9a3ecbe5ed12ab4d8e11ba873c2f11161202b945</t>
+          <t>sha256:ae252be0da5024d144ae862cddaa9a71102050f2b43ed244fc8b29d1425bb901</t>
         </is>
       </c>
     </row>
@@ -2014,10 +2026,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -2262,12 +2274,24 @@
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="S2" s="5" t="inlineStr"/>
-      <c r="T2" s="5" t="inlineStr"/>
-      <c r="U2" s="5" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d4/semantic_repair_browser.mjs</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>test_cmsr_d4_001</t>
+        </is>
+      </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
           <t>mock</t>
@@ -2291,7 +2315,7 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:4f53cda18c2baa0c0354bb5f9a3ecbe5ed12ab4d8e11ba873c2f11161202b945</t>
+          <t>sha256:9c83a2f64a371eae2149c016d79e511b8ef0d9171af65018c508fc676fe6d085</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: allow JSON imports in local tool fast path
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -723,7 +723,7 @@
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="29" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="42" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
@@ -1460,12 +1460,14 @@
       <c r="M6" s="5" t="inlineStr">
         <is>
           <t>1. Execute assignment, print and final_answer using an approved official tool. =&gt; The value, logs and final flag match the local interpreter.
-2. Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+2. Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.
+3. Import json or loads/dumps using direct and aliased forms, parse an official tool result, serialize it with nested JSON calls and reuse aliases in later steps. =&gt; Values and logs match the real local interpreter with no ordinary executor.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Factory acquisition and warm-up counts are zero.
+JSON loads/dumps and their import aliases work across steps without Docker.
 The wrapped tool is called once and final_answer returns the saved result.
 Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request.</t>
         </is>
@@ -1477,7 +1479,7 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Factory acquisition and warm-up counts are zero.","The wrapped tool is called once and final_answer returns the saved result.","Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request."],"inputs":["Simple official tool steps and final answers never acquire Docker"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+          <t>{"assertions":["Factory acquisition and warm-up counts are zero.","JSON loads/dumps and their import aliases work across steps without Docker.","The wrapped tool is called once and final_answer returns the saved result.","Official aidp_search uses its existing allowed KDS scope and emits real tool events without Docker, including an empty permission scope with no provider request."],"inputs":["Simple official tool steps and final answers never acquire Docker"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr"/>
@@ -1489,19 +1491,25 @@
       <c r="S6" s="5" t="inlineStr">
         <is>
           <t>pytest
+pytest
+pytest
 pytest</t>
         </is>
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_tool_fastpath.py
-test/automation/d1/test_tool_fastpath_aidp.py</t>
+test/automation/d1/test_tool_fastpath_aidp.py
+test/automation/d1/test_tool_fastpath_json.py
+test/automation/d1/test_tool_fastpath_json.py</t>
         </is>
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
           <t>test_tfp_d1_001
-test_tfp_d1_001_aidp</t>
+test_tfp_d1_001_aidp
+test_tfp_d1_001_json
+test_tfp_d1_001_json_tool_results</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
@@ -1518,12 +1526,12 @@
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
-          <t>sha256:f49d99ec8a0bad9223bdd15df090912a0a2c67816b5857d6add0a9fbd42f851c</t>
+          <t>sha256:7891191daf2e4c1801ad541da60c43d9185628c1903be8cc4fd92d5ed179b8c0</t>
         </is>
       </c>
       <c r="AA6" s="5" t="inlineStr">
         <is>
-          <t>sha256:01d39055c92bd0c0fe6e4360ed1345a6eae93173d20da7f1fea830c15a61839e</t>
+          <t>sha256:440cb5a48b22ca2a72b2000ec4d0af860f20a59b80d96212595e5b6d5bf92837</t>
         </is>
       </c>
     </row>
@@ -1590,13 +1598,15 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>1. Submit a tool call followed by an import, an unapproved call or a bare data expression outside assignment and call arguments. =&gt; The whole step is delegated before any local call.
-2. An aidp_search step followed by ordinary code makes no provider request before whole-step delegation. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+          <t>1. Submit a tool call followed by an unapproved import, an unapproved call or a bare data expression outside assignment and call arguments. =&gt; The whole step is delegated before any local call.
+2. An aidp_search step followed by ordinary code makes no provider request before whole-step delegation. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.
+3. Submit JSON imports and tool calls mixed with file-oriented JSON operations, unapproved members, wildcard/relative/dynamic imports or ordinary Python syntax. =&gt; Delegate the entire source before executing any local import or tool.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
           <t>Mixed code is passed once to the original executor.
+Admitted JSON statements do not cause partial execution of rejected mixed steps.
 No approved tool is called by the fast path before delegation.
 An aidp_search step followed by ordinary code makes no provider request before whole-step delegation.</t>
         </is>
@@ -1608,7 +1618,7 @@
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Mixed code is passed once to the original executor.","No approved tool is called by the fast path before delegation.","An aidp_search step followed by ordinary code makes no provider request before whole-step delegation."],"inputs":["Full-step admission prevents partial local execution"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+          <t>{"assertions":["Mixed code is passed once to the original executor.","Admitted JSON statements do not cause partial execution of rejected mixed steps.","No approved tool is called by the fast path before delegation.","An aidp_search step followed by ordinary code makes no provider request before whole-step delegation."],"inputs":["Full-step admission prevents partial local execution"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr"/>
@@ -1620,19 +1630,22 @@
       <c r="S7" s="5" t="inlineStr">
         <is>
           <t>pytest
+pytest
 pytest</t>
         </is>
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
           <t>test/automation/d1/test_tool_fastpath.py
-test/automation/d1/test_tool_fastpath_aidp.py</t>
+test/automation/d1/test_tool_fastpath_aidp.py
+test/automation/d1/test_tool_fastpath_json.py</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
           <t>test_tfp_d1_002
-test_tfp_d1_002_aidp</t>
+test_tfp_d1_002_aidp
+test_tfp_d1_002_json</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
@@ -1649,12 +1662,12 @@
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
-          <t>sha256:45bd2b9559253a21e4b96e995b91daa065ff8f9ea28bf3c3908b9756b5791782</t>
+          <t>sha256:97f3565d985b576df5e9a23518cb625ca0d4796b4bf0378a8f1773d4f38073e7</t>
         </is>
       </c>
       <c r="AA7" s="5" t="inlineStr">
         <is>
-          <t>sha256:01d39055c92bd0c0fe6e4360ed1345a6eae93173d20da7f1fea830c15a61839e</t>
+          <t>sha256:8fdbcb9d596383c8e5a55a84bc25f9f9033ad33cad2d2a91bc362ed09c3f4446</t>
         </is>
       </c>
     </row>
@@ -1722,13 +1735,15 @@
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>1. Produce aliased user containers and a tool result, then submit ordinary code. =&gt; One executor is initialized and receives the user namespace.
-2. Submit another approved step. =&gt; The initialized executor is reused.</t>
+2. Submit another approved step. =&gt; The initialized executor is reused.
+3. Import json/loads/dumps with aliases, save parsed data and then activate ordinary code that uses those aliases. Include prior data names replaced by imports. =&gt; Recreate the actual imports once before ordinary code; migrate only user data and preserve references without replaying prior tools.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
           <t>Values and shared container references survive migration.
 Internal interpreter state and tool objects are not migrated.
+JSON module/function objects are excluded; actual imported aliases are recreated.
 The factory is called once.</t>
         </is>
       </c>
@@ -1739,7 +1754,7 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Values and shared container references survive migration.","Internal interpreter state and tool objects are not migrated.","The factory is called once."],"inputs":["Promotion preserves user values and remains sticky"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+          <t>{"assertions":["Values and shared container references survive migration.","Internal interpreter state and tool objects are not migrated.","JSON module/function objects are excluded; actual imported aliases are recreated.","The factory is called once."],"inputs":["Promotion preserves user values and remains sticky"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr"/>
@@ -1750,17 +1765,23 @@
       </c>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>pytest</t>
+          <t>pytest
+pytest
+pytest</t>
         </is>
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>test/automation/d1/test_tool_fastpath.py</t>
+          <t>test/automation/d1/test_tool_fastpath.py
+test/automation/d1/test_tool_fastpath_json.py
+test/automation/d1/test_tool_fastpath_json.py</t>
         </is>
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>test_tfp_d1_003</t>
+          <t>test_tfp_d1_003
+test_tfp_d1_003_json
+test_tfp_d1_003_json_replaced_binding</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
@@ -1777,12 +1798,12 @@
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
-          <t>sha256:78c3f112432755e552f23bdb788339f518f550d911228d013071fc2c932db42d</t>
+          <t>sha256:f1bc59890f25b5b66c1816e60700a0c3fd04f3b3c72f42e1538ed10f90eee37c</t>
         </is>
       </c>
       <c r="AA8" s="5" t="inlineStr">
         <is>
-          <t>sha256:fba0f34909d32b214bd0a02edc0f4c28eaf34e88e682b3977a2f5a6ea22a64cb</t>
+          <t>sha256:0c084ac84eae8f370c9130fd6f12f32c7f66727ea8be97e748d131d09fc6a158</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1934,7 @@
       </c>
       <c r="AA9" s="5" t="inlineStr">
         <is>
-          <t>sha256:01d39055c92bd0c0fe6e4360ed1345a6eae93173d20da7f1fea830c15a61839e</t>
+          <t>sha256:d51fb991cae4fea09f646ea0e34dc9914cba84cd3a5834c2494eb30c77e5bc3c</t>
         </is>
       </c>
     </row>
@@ -1981,12 +2002,15 @@
       <c r="M10" s="5" t="inlineStr">
         <is>
           <t>1. Fail an approved tool, close an unused wrapper, fail workspace or variable initialization and cancel during acquisition. =&gt; No failed call is replayed and acquired resources close once.
-2. AIDP provider errors propagate without acquiring or replaying through Docker. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.</t>
+2. AIDP provider errors propagate without acquiring or replaying through Docker. =&gt; The existing AIDP authorization and complete-step routing contract is preserved.
+3. Fail JSON parsing between admitted imports, then reuse completed imports or activate ordinary code. Fail or cancel import restoration during activation. =&gt; Do not replay errors, tools or unfinished imports; preserve actual bindings and release acquired executors exactly once.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
           <t>Local errors do not trigger remote replay.
+JSON errors retain only executed imports and never acquire an executor by themselves.
+Failed or cancelled import restoration releases the acquired executor without replay.
 Cleanup is idempotent.
 Cancellation before execution prevents tool calls and releases acquired resources.
 AIDP provider errors propagate without acquiring or replaying through Docker.</t>
@@ -2000,7 +2024,7 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>{"assertions":["Local errors do not trigger remote replay.","Cleanup is idempotent.","Cancellation before execution prevents tool calls and releases acquired resources.","AIDP provider errors propagate without acquiring or replaying through Docker."],"inputs":["Exceptions, cancellation and cleanup are safe"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
+          <t>{"assertions":["Local errors do not trigger remote replay.","JSON errors retain only executed imports and never acquire an executor by themselves.","Failed or cancelled import restoration releases the acquired executor without replay.","Cleanup is idempotent.","Cancellation before execution prevents tool calls and releases acquired resources.","AIDP provider errors propagate without acquiring or replaying through Docker."],"inputs":["Exceptions, cancellation and cleanup are safe"],"unit_boundary":"Restricted AST admission, real LocalPythonExecutor and NexentAgent executor lifecycle"}</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr"/>
@@ -2013,6 +2037,9 @@
         <is>
           <t>pytest
 pytest
+pytest
+pytest
+pytest
 pytest</t>
         </is>
       </c>
@@ -2020,14 +2047,20 @@
         <is>
           <t>test/automation/d1/test_tool_fastpath.py
 test/automation/d1/test_tool_fastpath.py
-test/automation/d1/test_tool_fastpath_aidp.py</t>
+test/automation/d1/test_tool_fastpath_aidp.py
+test/automation/d1/test_tool_fastpath_json.py
+test/automation/d1/test_tool_fastpath_json.py
+test/automation/d1/test_tool_fastpath_json.py</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
           <t>test_tfp_d1_005
 test_tfp_d1_005_deferred_setup
-test_tfp_d1_005_aidp</t>
+test_tfp_d1_005_aidp
+test_tfp_d1_005_json_error
+test_tfp_d1_005_json_rebinding_error
+test_tfp_d1_005_json_restore_failure</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
@@ -2044,12 +2077,12 @@
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
-          <t>sha256:f9b9a844e326fc8cac16cb7fa2c69d2ea2f5604696c678c814dfa2ff0058d915</t>
+          <t>sha256:e1415a3a6af4da41671b4363b8c4b4eba52a6dd47b4b4296227c3f43d660734d</t>
         </is>
       </c>
       <c r="AA10" s="5" t="inlineStr">
         <is>
-          <t>sha256:e263aa60250b6329f8943aaa6a2f8f0be1b27c3a8dcdfc7364eff56c8ededcaa</t>
+          <t>sha256:9fa401f941bf919e6f8136c5e4ba60fa481f2c824e7b1c2b54b555ff9746b4fd</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2226,7 @@
       </c>
       <c r="AA11" s="5" t="inlineStr">
         <is>
-          <t>sha256:071883550d50b75dd6588a75d883d5af51a92b6edadbf1c02b30412179705beb</t>
+          <t>sha256:56280e4bb05195c39eb91616119beadf4479255a48d8db2a5a23db734b9f2371</t>
         </is>
       </c>
     </row>
@@ -3427,9 +3460,9 @@
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -3762,13 +3795,15 @@
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>1. Submit attributes, imports, alias calls, unpacking, loops and reserved-variable assignments, including initial variables that shadow tool or framework call names. =&gt; All are rejected before execution.</t>
+          <t>1. Submit arbitrary attributes/imports, alias calls, unpacking, loops and reserved-variable assignments, including initial variables that shadow tool or framework call names. =&gt; All are rejected before execution.
+2. Forge JSON modules/functions through initial variables or change an admitted binding; use JSON file operations, dynamic callbacks, wildcard imports and reserved alias names. =&gt; Reject the entire step with no local import, callback or tool effects.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Zero local tool calls for all rejected inputs.
-The full source is delegated unchanged.</t>
+The full source is delegated unchanged.
+Only exact admitted JSON loads/dumps bindings qualify; shadowed bindings never invoke locally.</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
@@ -3789,17 +3824,23 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>pytest</t>
+          <t>pytest
+pytest
+pytest</t>
         </is>
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>test/automation/d5/test_tool_fastpath_risks.py</t>
+          <t>test/automation/d5/test_tool_fastpath_risks.py
+test/automation/d5/test_tool_fastpath_json_risks.py
+test/automation/d5/test_tool_fastpath_json_risks.py</t>
         </is>
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>test_tfp_d5_001</t>
+          <t>test_tfp_d5_001
+test_tfp_d5_001_json_syntax
+test_tfp_d5_001_json_identity</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
@@ -3816,12 +3857,12 @@
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>sha256:cad74b7982db6a898f9267891d908d5e4a026fff456b4e16172e26fa1f499f08</t>
+          <t>sha256:a95f4672fd09d8d82014f5b21de9850d7cf8d4dd7eb6c5bea2f8062f675ed512</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>sha256:6af5717e8cd49952880712aeb98f89e5242c74430374ce491d472e1f80f687cc</t>
+          <t>sha256:4fd0bf1be9902c93374ec9c0e5145b2676d332ac3c2b7f8c70c62707af221a07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(agent): tolerate incomplete thinking prefixes without raw protocol finals
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_D5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_D2'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_D5'!$A$1:$AA$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_D5'!$A$1:$AA$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -646,8 +646,50 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Thinking prefix compatibility</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Reasoning markup does not block valid actions or authorize raw final answers.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001
+TPC-RULE-002
+TPC-RULE-003</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>D1
+D3
+D4
+D5</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>{"requirement_ids":["TPC-001"],"spec_path":"nexent-doc/docs/Developing/codeagent-explicit-termination/changes/codeagent-think-prefix-compatibility/proposal.md"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -658,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1351,8 +1393,769 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D1-001</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Compatible thinking prefixes yield the exact executable action</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Compatible thinking prefixes yield the exact executable action</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>1. Classify plain, paired-plus-narration, orphan, unclosed, repeated and nested thinking prefixes before complete code and run actions. =&gt; Every result is an executable action with the exact Python body.</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>All compatible prefixes accepted.</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Prefix text is never executed.</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Exact executable body and legacy flag."],"inputs":["prefix matrix","code/run envelopes"],"unit_boundary":"classify_model_output"}</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_think_prefix_compatibility.py</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d1_001</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:4f391cdcc5d8afa20a295a40d9739667d853c3099df0248d511947163488a722</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:80150f5dbffa58305e628681d5dd93c39d59d2d701854cc6967112e494836fab</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D1-002</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001
+TPC-RULE-003</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Skill reads execute rather than finalize at first and third generations</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Skill reads execute rather than finalize at first and third generations</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>1. Run complete skill read under every compatible prefix with prior error counters zero and two. =&gt; One read executes; its result is an observation; no final answer is returned.</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Exactly one tool effect per action.
+Model attempt commits.</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>No raw final answer.
+No extra model request.</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Skill call count one.","ActionOutput.is_final_answer false.","Accepted attempt commits without rollback."],"inputs":["prefix matrix","prior errors zero/two"],"unit_boundary":"CoreAgent._step_stream and Python executor boundary"}</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_think_prefix_compatibility.py</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d1_002</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" s="5" t="inlineStr"/>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:bf3161e59bf8555b8eca4685fd76b62450ac76b189b1f54db8a6d943022475ed</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:80150f5dbffa58305e628681d5dd93c39d59d2d701854cc6967112e494836fab</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D1-003</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001
+TPC-RULE-002</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Malformed actions retain structural rejection</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Malformed actions retain structural rejection</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>1. Classify invalid Python, empty/unclosed action, inter-block text, trailing text, unknown tags and truncated output. =&gt; Protocol error occurs; no executor is called.</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Invalid action bodies and boundaries remain rejected.</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>No execution of invalid code.</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Expected stable protocol-error reason."],"inputs":["invalid action/control matrix","length finish reason"],"unit_boundary":"classify_model_output"}</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_think_prefix_compatibility.py</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d1_003</t>
+        </is>
+      </c>
+      <c r="V8" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W8" s="5" t="inlineStr"/>
+      <c r="X8" s="5" t="inlineStr"/>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z8" s="5" t="inlineStr">
+        <is>
+          <t>sha256:100d35b68a2e856ce77afbea76a04f64cced55b7c6427ad4b682ff63a5512759</t>
+        </is>
+      </c>
+      <c r="AA8" s="5" t="inlineStr">
+        <is>
+          <t>sha256:80150f5dbffa58305e628681d5dd93c39d59d2d701854cc6967112e494836fab</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D1-004</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-002</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Thinking-only and invalid marked output never use exhausted raw final</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Thinking-only and invalid marked output never use exhausted raw final</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>1. Run thinking-only and malformed action or final outputs with two prior protocol errors. =&gt; The attempt rolls back and no raw final is accepted.
+2. Run eligible complete plain text at exhaustion. =&gt; Existing raw candidate remains accepted.</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Marked failures cannot finalize.
+Eligible plain text keeps existing fallback.</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>No invalid action final.
+No reasoning final.</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Failed attempt rollback.","No executor call on invalid output.","Plain raw fallback preserved."],"inputs":["marked output","plain text","error count two"],"unit_boundary":"CoreAgent._accept_exhausted_raw_output and _step_stream"}</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_think_prefix_compatibility.py</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d1_004</t>
+        </is>
+      </c>
+      <c r="V9" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr"/>
+      <c r="X9" s="5" t="inlineStr"/>
+      <c r="Y9" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z9" s="5" t="inlineStr">
+        <is>
+          <t>sha256:f2504ffd5633cd2255b5dbbd3f2265227f687a753a12a0145d193b141a18ef32</t>
+        </is>
+      </c>
+      <c r="AA9" s="5" t="inlineStr">
+        <is>
+          <t>sha256:80150f5dbffa58305e628681d5dd93c39d59d2d701854cc6967112e494836fab</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D1-005</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001
+TPC-RULE-002</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Ordinary explicit finals tolerate thinking prefix and keep boundaries</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Ordinary explicit finals tolerate thinking prefix and keep boundaries</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>1. Classify compatible prefix before valid ordinary final envelope. =&gt; Only the payload is ExplicitFinalAnswer.
+2. Classify duplicates, incomplete envelopes, suffix text and specialized prefixed envelopes. =&gt; Protocol errors remain.</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Ordinary terminal prefix accepted.
+Specialized exact-envelope behavior retained.</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>No prefix in terminal payload.
+No malformed final accepted.</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Exact final payload.","Malformed and specialized prefixed forms reject."],"inputs":["prefix matrix","final envelope matrix","final_envelope protocol"],"unit_boundary":"classify_model_output terminal branch"}</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_think_prefix_compatibility.py</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d1_005</t>
+        </is>
+      </c>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr"/>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>sha256:33d570993c8638b85cd01d13e5fde4178f0bae8302be5d3108471cb7fc0d257b</t>
+        </is>
+      </c>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>sha256:80150f5dbffa58305e628681d5dd93c39d59d2d701854cc6967112e494836fab</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D1-006</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Python data containing protocol-like tags is preserved</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>SDK-UT</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Python data containing protocol-like tags is preserved</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>1. Classify actions whose strings/comments contain think and code markers. =&gt; Python data remains unchanged and executable.</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Only outer reasoning prefix is normalized.</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>No global tag replacement in action or final data.</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Exact code body retained."],"inputs":["Python literal/comment protocol-like text"],"unit_boundary":"classify_model_output Python data boundaries"}</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_think_prefix_compatibility.py</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d1_006</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W11" s="5" t="inlineStr"/>
+      <c r="X11" s="5" t="inlineStr"/>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z11" s="5" t="inlineStr">
+        <is>
+          <t>sha256:b76ef5ea9a602bd23ed01d075a888e34440cd8c9d6585726a2e366975f398087</t>
+        </is>
+      </c>
+      <c r="AA11" s="5" t="inlineStr">
+        <is>
+          <t>sha256:80150f5dbffa58305e628681d5dd93c39d59d2d701854cc6967112e494836fab</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA5"/>
+  <autoFilter ref="A1:AA11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1663,7 +2466,7 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:570d7db5b7480c6b3a3a3adcc953158f7c496e44a79e90ad1ca3a4df676d573f</t>
+          <t>sha256:f8f1bc3e7a01d6ffd739d9fbe695e28533e4c410847a09b6405a7dbd4c2e948a</t>
         </is>
       </c>
     </row>
@@ -1679,7 +2482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1699,10 +2502,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="42" customWidth="1" min="21" max="21"/>
     <col width="17" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -1981,8 +2784,154 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D3-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-001
+TPC-RULE-003</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Deployed skill read completes with explicit final and persisted evidence</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>AGENT-IT</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Deployed skill read completes with explicit final and persisted evidence</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Disposable Nexent deployment, authorized skill and controlled provider are available.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Drive controlled think prefix then skill-read action through deployed Agent. =&gt; Read executes once and returns skill text.
+2. Return a separate explicit final and reload history. =&gt; Exactly one final payload and one read result are persisted.
+3. Exhaust three malformed marked responses without an executable action. =&gt; No skill effect or raw protocol final is emitted or stored.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Runtime executes the skill read.
+History matches committed stream.
+Malformed marked exhaustion does not execute or become a raw final.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No unexecuted action final.
+No duplicate tool effects.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"cleanup":["Remove test conversation and provider fixture."],"integration_boundary":["Provider to classifier","Executor to skill tool","Observer to SSE/history"],"observations":["Raw content and parser classification","Skill tool effect","Final source and stored units"]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["model-provider"]},{"name":"real_smoke","required_services":["model-provider"]}]}</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>pytest
+pytest
+pytest</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d3/test_think_prefix_runtime.py
+test/automation/d3/test_think_prefix_runtime.py
+test/automation/d3/test_think_prefix_runtime.py</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d3_001_skill_executes_once_and_history_matches
+test_tpc_d3_001_marked_exhaustion_never_executes_or_finalizes
+test_tpc_d3_001_real_model_reads_skill</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock
+real_smoke</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>model-provider</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:2de8f6fa8b9e8b2e53318f71e08dccbb4cbe6e95935069f88ca84a3eebb66f0c</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:aed01ec6f1542f3267c7c65eb7c60830b2150eb4fd123fa4c174e2b729753149</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1993,7 +2942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2013,10 +2962,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -2294,8 +3243,143 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D4-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-003</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Skill journey remains correct after browser reload</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Skill journey remains correct after browser reload</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Disposable Nexent deployment, authorized skill and controlled provider are available.
+Fresh test tenant has default memory enabled and no embedding model; dismiss its warning without changing settings.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Open test Agent and request a skill-based check. =&gt; Skill read and result are visible.
+2. Wait for final, reload the workbench, then reopen the saved conversation from its sidebar entry. =&gt; Final contains the result, not the unexecuted action.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Skill check business result is visible after refresh.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No raw action final.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"actor":"Tenant test user","failure_evidence":["Sanitized browser trace and failed assertion screenshot."],"final_business_result":["Completed skill check with preserved tool result and validated final."],"journey":["Open Agent","Submit check","Observe skill execution","Reload saved conversation"]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>{"profiles":[{"name":"mock","required_services":["model-provider"]}]}</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d4/think_prefix_browser.mjs</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d4_001</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>model-provider</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:a4396130631c96c17607bc377500d220995c93f701be28bdfbb7c96d2c66556c</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:ed5c9e72e1af0ac98d23c22f314b32d163311a4e3bbca87dd9d77997576aedc8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2306,7 +3390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2326,10 +3410,10 @@
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
@@ -2599,8 +3683,137 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-D5-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-001</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>TPC-RULE-002
+TPC-RULE-003</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Protocol exhaustion and truncation never authorize unsafe replay or final</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>RELIABILITY</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Protocol exhaustion and truncation never authorize unsafe replay or final</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Isolated strict ordinary CodeAgent with a controlled model and authorized skill-read tool.</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>{"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>1. Run two rejected actions then a third malformed action or length-truncated action. =&gt; No executor call or raw final occurs.
+2. Run a valid compatible skill action after two rejections. =&gt; Exactly one execution commits, with no replay.</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Invalid third attempt never finalizes.
+Valid action executes exactly once.</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No invalid execution.
+No tool replay.</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>{"condition":["Prior error count two","Malformed/truncated third generation","Valid third compatible action"],"metrics":["Executor invocation count","Invalid raw final count","Accepted attempt count"],"recovery_expectations":["Valid actions recover; invalid exhausted responses stay bounded failures."],"risk":"Protocol repair can skip skills or publish unexecuted actions as final answers.","risk_type":"RELIABILITY","thresholds":["Zero executor invocations for invalid output","Zero invalid raw final answers","Exactly one invocation for valid action"]}</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d5/test_think_prefix_reliability.py</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>test_tpc_d5_001</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:a56e85d3e652c38805e425c416214927664a2155d0836a31251fb4a10531659d</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>sha256:a04e4124b9b4a97aaae836e61e9ccf12512e97957c4c232e3d52c7a593565ed9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA2"/>
+  <autoFilter ref="A1:AA3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: consolidate model management services
</commit_message>
<xml_diff>
--- a/test/generated/Nexent_测试基线.xlsx
+++ b/test/generated/Nexent_测试基线.xlsx
@@ -16,8 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_D5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_功能清单'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_D1'!$A$1:$AA$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_D2'!$A$1:$AA$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_D3'!$A$1:$AA$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_D4'!$A$1:$AA$2</definedName>
@@ -551,11 +551,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -646,8 +646,46 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-001</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Model service ownership and preserved contracts</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Model services and utilities have one Management implementation with shared immutable contracts.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-RULE-001
+MSRF-RULE-002</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>{"requirement_ids":["MSRF-001"],"spec_path":"nexent-doc/docs/Developing/four-service-runtime-decoupling/changes/model-service-refactor/proposal.md"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -658,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1351,8 +1389,263 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-D1-001</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-001</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-001</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-RULE-001</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Model implementation has one bounded canonical location</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>BE-UT</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Verify canonical locations and an acyclic internal import graph.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Use repository Python sources without external services.</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>{"max_physical_lines":1500,"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>1. Inspect model sources and all backend SDK and test imports. =&gt; Canonical files exist and obsolete imports and duplicate implementations are absent.
+2. Traverse model internal imports including function-local imports. =&gt; No cycle connects provider health and probe.</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Every model code file is at most 1500 lines.
+All internal dependencies are acyclic.</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>No database or provider connection occurs during source inspection.</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Required canonical modules exist.","Obsolete modules are absent.","Import graph has no cycle.","Names depends only on standard library."],"inputs":["Repository Python source files"],"unit_boundary":"Model source ownership and dependency graph"}</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_model_service_refactor.py</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>test_msrf_d1_001</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:c9f190fbea88ebaf8a22dd6172145101c7cdf404be72b1d36e4968d81a44ee32</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>sha256:06eba556ec2713839a39898941ae1c72d98f1a1a43d282e30709d2cff5c7145f</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-D1-002</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-001</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-001</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>MSRF-RULE-002</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Relocated model methods and shared types preserve their contracts</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>BE-UT</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>automated</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Compare signatures to the develop baseline and check immutable result defaults.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Use the captured develop signature fixture and pure contracts.</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>{"configurations":["empty name","repository qualified name","legacy modelName"],"profile":"mock"}</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>1. Compare canonical function signatures to baseline declarations. =&gt; Arguments defaults return annotations and async declarations match.
+2. Construct model descriptors and capacity results and format model names. =&gt; Defaults enum values and name fallback behavior match the preserved contract.</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>All captured signatures match.
+Shared dataclasses remain frozen.
+Name formatting preserves legacy fields.</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>No model client database or telemetry initialization is required for contracts or names.</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>{"assertions":["Public signatures are unchanged.","Contract defaults and enum values match.","Dataclasses reject mutation.","Pure helpers use no business imports."],"inputs":["Baseline signatures","Empty and legacy model name dictionaries"],"unit_boundary":"Public model signatures immutable contracts and pure name helpers"}</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>test/automation/d1/test_model_service_refactor.py</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>test_msrf_d1_002</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>mock</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" s="5" t="inlineStr"/>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>校验通过</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:370fa658828de25e16474d3dd8cfd8047f7e21e8bb5b1f8411a5d69ce2e13d58</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>sha256:06eba556ec2713839a39898941ae1c72d98f1a1a43d282e30709d2cff5c7145f</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA5"/>
+  <autoFilter ref="A1:AA7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1663,7 +1956,7 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>sha256:570d7db5b7480c6b3a3a3adcc953158f7c496e44a79e90ad1ca3a4df676d573f</t>
+          <t>sha256:f8f1bc3e7a01d6ffd739d9fbe695e28533e4c410847a09b6405a7dbd4c2e948a</t>
         </is>
       </c>
     </row>

</xml_diff>